<commit_message>
chore(frontend): rebuild the demo report on the regenerated kit
python -m arm_web build-demo with PDFium and Tesseract 5.5.2. The report
was last built by the prototype. Structure, discrepancies and summary are
the same; title blocks of scans score 0.625 instead of 0.375, requirement
parameters F1 0.963 instead of 0.975.
</commit_message>
<xml_diff>
--- a/frontend/public/demo/report.xlsx
+++ b/frontend/public/demo/report.xlsx
@@ -484,7 +484,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-10-20T16:00:34+00:00</t>
+          <t>2026-10-21T08:59:33+00:00</t>
         </is>
       </c>
     </row>
@@ -2627,9 +2627,21 @@
         </is>
       </c>
       <c r="D5" s="3" t="n"/>
-      <c r="E5" s="3" t="n"/>
-      <c r="F5" s="3" t="n"/>
-      <c r="G5" s="3" t="n"/>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>1,2</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>1:1</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>О1</t>
+        </is>
+      </c>
       <c r="H5" s="3" t="n"/>
       <c r="I5" s="3" t="n"/>
       <c r="J5" s="3" t="n"/>
@@ -3034,7 +3046,11 @@
           <t>0,22</t>
         </is>
       </c>
-      <c r="F13" s="3" t="n"/>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>1:1</t>
+        </is>
+      </c>
       <c r="G13" s="3" t="inlineStr">
         <is>
           <t>О1</t>
@@ -4242,7 +4258,7 @@
       </c>
       <c r="M19" s="3" t="inlineStr">
         <is>
-          <t>Покрытие Хим.Окс.прм</t>
+          <t>. Покрытие Хим.Окс.прм.</t>
         </is>
       </c>
       <c r="N19" s="3" t="inlineStr">
@@ -4269,21 +4285,15 @@
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>IT14</t>
+          <t>Неуказанные отклонения</t>
         </is>
       </c>
       <c r="E20" s="3" t="n"/>
       <c r="F20" s="3" t="n"/>
       <c r="G20" s="3" t="n"/>
       <c r="H20" s="3" t="n"/>
-      <c r="I20" s="3" t="inlineStr">
-        <is>
-          <t>h14</t>
-        </is>
-      </c>
-      <c r="J20" s="3" t="n">
-        <v>14</v>
-      </c>
+      <c r="I20" s="3" t="n"/>
+      <c r="J20" s="3" t="n"/>
       <c r="K20" s="3" t="inlineStr">
         <is>
           <t>да</t>
@@ -4292,7 +4302,7 @@
       <c r="L20" s="3" t="inlineStr"/>
       <c r="M20" s="3" t="inlineStr">
         <is>
-          <t>Неуказанные предельные отклонения размеров: Н14, h14, +IT14/2</t>
+          <t>Неуказанные предельные отклонения размеров: Н14, 114, +1T14/2.</t>
         </is>
       </c>
       <c r="N20" s="3" t="inlineStr">
@@ -6464,7 +6474,7 @@
       <c r="L62" s="3" t="inlineStr"/>
       <c r="M62" s="3" t="inlineStr">
         <is>
-          <t>Q50H9</t>
+          <t>@50H9</t>
         </is>
       </c>
       <c r="N62" s="3" t="inlineStr">
@@ -6514,7 +6524,7 @@
       <c r="L63" s="3" t="inlineStr"/>
       <c r="M63" s="3" t="inlineStr">
         <is>
-          <t>Ка 3,2</t>
+          <t>Ва 3,2</t>
         </is>
       </c>
       <c r="N63" s="3" t="inlineStr">
@@ -8324,7 +8334,7 @@
       </c>
       <c r="D24" s="3" t="inlineStr">
         <is>
-          <t>Покрытие Хим.Окс.прм</t>
+          <t>. Покрытие Хим.Окс.прм.</t>
         </is>
       </c>
       <c r="E24" s="3" t="inlineStr">
@@ -10116,7 +10126,7 @@
       </c>
       <c r="H22" s="3" t="inlineStr">
         <is>
-          <t>Файл повреждён или не открывается: Failed to open stream</t>
+          <t>Файл повреждён или не открывается: Failed to load document (PDFium: Data format error).</t>
         </is>
       </c>
       <c r="I22" s="3" t="inlineStr"/>
@@ -10489,7 +10499,7 @@
       <c r="D13" s="3" t="n"/>
       <c r="E13" s="3" t="n"/>
       <c r="F13" s="3" t="n">
-        <v>0.9330000000000001</v>
+        <v>1</v>
       </c>
       <c r="G13" s="3" t="n">
         <v>15</v>
@@ -10510,7 +10520,7 @@
       <c r="D14" s="3" t="n"/>
       <c r="E14" s="3" t="n"/>
       <c r="F14" s="3" t="n">
-        <v>0.867</v>
+        <v>1</v>
       </c>
       <c r="G14" s="3" t="n">
         <v>15</v>
@@ -10531,7 +10541,7 @@
       <c r="D15" s="3" t="n"/>
       <c r="E15" s="3" t="n"/>
       <c r="F15" s="3" t="n">
-        <v>0.9330000000000001</v>
+        <v>1</v>
       </c>
       <c r="G15" s="3" t="n">
         <v>15</v>
@@ -10636,7 +10646,7 @@
       <c r="D20" s="3" t="n"/>
       <c r="E20" s="3" t="n"/>
       <c r="F20" s="3" t="n">
-        <v>0.375</v>
+        <v>0.625</v>
       </c>
       <c r="G20" s="3" t="n">
         <v>16</v>
@@ -10654,13 +10664,13 @@
         </is>
       </c>
       <c r="C21" s="3" t="n">
-        <v>1</v>
+        <v>0.987</v>
       </c>
       <c r="D21" s="3" t="n">
-        <v>0.951</v>
+        <v>0.9389999999999999</v>
       </c>
       <c r="E21" s="3" t="n">
-        <v>0.975</v>
+        <v>0.963</v>
       </c>
       <c r="F21" s="3" t="n"/>
       <c r="G21" s="3" t="n">

</xml_diff>

<commit_message>
chore(frontend): rebuild the demo report on contract 1.2
Every discrepancy names its rule, every value has a status: 281 values
of the text layer are ok, the 12 values read by OCR are low_confidence,
the ones the web marked before. Apart from the new fields, the settings
hash and the times, the report is the same as before.
</commit_message>
<xml_diff>
--- a/frontend/public/demo/report.xlsx
+++ b/frontend/public/demo/report.xlsx
@@ -18,7 +18,7 @@
     <sheet name="Качество" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Расхождения'!$A$1:$I$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Расхождения'!$A$1:$J$10</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Дерево изделия'!$A$1:$J$27</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Основные надписи'!$A$1:$L$16</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Параметры'!$A$1:$N$79</definedName>
@@ -484,7 +484,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-10-21T15:39:15+00:00</t>
+          <t>2026-10-22T03:20:19+00:00</t>
         </is>
       </c>
     </row>
@@ -520,7 +520,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>e7b2b120a785f4893b1cb27c3c30fa6735edc8dca089b0ead5de44e7042498c8</t>
+          <t>63cd3acc4802cb6cb498201bf52b75da245da18316a4711d03f7e8b57b9a47bc</t>
         </is>
       </c>
     </row>
@@ -739,18 +739,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I10"/>
+  <dimension ref="A1:J10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
     <col width="26" customWidth="1" min="2" max="2"/>
-    <col width="11" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
-    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="6" max="6"/>
     <col width="20" customWidth="1" min="7" max="7"/>
-    <col width="40" customWidth="1" min="8" max="8"/>
+    <col width="20" customWidth="1" min="8" max="8"/>
     <col width="40" customWidth="1" min="9" max="9"/>
+    <col width="40" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -766,35 +767,40 @@
       </c>
       <c r="C1" s="2" t="inlineStr">
         <is>
+          <t>Правило</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
           <t>Важность</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="E1" s="2" t="inlineStr">
         <is>
           <t>Обозначение</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="F1" s="2" t="inlineStr">
         <is>
           <t>Описание</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="G1" s="2" t="inlineStr">
         <is>
           <t>Ожидалось</t>
         </is>
       </c>
-      <c r="G1" s="2" t="inlineStr">
+      <c r="H1" s="2" t="inlineStr">
         <is>
           <t>Фактически</t>
         </is>
       </c>
-      <c r="H1" s="2" t="inlineStr">
+      <c r="I1" s="2" t="inlineStr">
         <is>
           <t>Документы</t>
         </is>
       </c>
-      <c r="I1" s="2" t="inlineStr">
+      <c r="J1" s="2" t="inlineStr">
         <is>
           <t>Источник</t>
         </is>
@@ -811,31 +817,36 @@
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
+          <t>B1.MISSING.001</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
           <t>Высокая</t>
         </is>
       </c>
-      <c r="D2" s="3" t="inlineStr">
+      <c r="E2" s="3" t="inlineStr">
         <is>
           <t>АРМ.303411.103</t>
         </is>
       </c>
-      <c r="E2" s="3" t="inlineStr">
+      <c r="F2" s="3" t="inlineStr">
         <is>
           <t>Чертёж детали АРМ.303411.103 «Втулка» указан в спецификации АРМ.303411.100, но в комплекте не найден</t>
         </is>
       </c>
-      <c r="F2" s="3" t="inlineStr">
+      <c r="G2" s="3" t="inlineStr">
         <is>
           <t>АРМ.303411.103</t>
         </is>
       </c>
-      <c r="G2" s="3" t="n"/>
-      <c r="H2" s="3" t="inlineStr">
+      <c r="H2" s="3" t="n"/>
+      <c r="I2" s="3" t="inlineStr">
         <is>
           <t>Спецификации/АРМ.303411.100 Корпус в сборе.pdf</t>
         </is>
       </c>
-      <c r="I2" s="3" t="inlineStr">
+      <c r="J2" s="3" t="inlineStr">
         <is>
           <t>Спецификации/АРМ.303411.100 Корпус в сборе.pdf, стр. 1</t>
         </is>
@@ -852,27 +863,32 @@
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
+          <t>B1.SPEC.001</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
           <t>Высокая</t>
         </is>
       </c>
-      <c r="D3" s="3" t="inlineStr">
+      <c r="E3" s="3" t="inlineStr">
         <is>
           <t>АРМ.303411.300</t>
         </is>
       </c>
-      <c r="E3" s="3" t="inlineStr">
+      <c r="F3" s="3" t="inlineStr">
         <is>
           <t>Сборочная единица АРМ.303411.300 указана в спецификации, но её спецификация в комплекте отсутствует; сборочный чертёж есть, состав раскрыть невозможно</t>
         </is>
       </c>
-      <c r="F3" s="3" t="n"/>
       <c r="G3" s="3" t="n"/>
-      <c r="H3" s="3" t="inlineStr">
+      <c r="H3" s="3" t="n"/>
+      <c r="I3" s="3" t="inlineStr">
         <is>
           <t>Чертежи/АРМ.303411.300 СБ.pdf</t>
         </is>
       </c>
-      <c r="I3" s="3" t="inlineStr">
+      <c r="J3" s="3" t="inlineStr">
         <is>
           <t>Спецификации/АРМ.303411.000 Редуктор колёсный.pdf, стр. 1</t>
         </is>
@@ -889,31 +905,36 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
+          <t>B1.MISSING.001</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
           <t>Высокая</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="E4" s="3" t="inlineStr">
         <is>
           <t>АРМ.303411.004</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="F4" s="3" t="inlineStr">
         <is>
           <t>Чертёж детали АРМ.303411.004 «Прокладка» указан в спецификации АРМ.303411.000, но в комплекте не найден</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="G4" s="3" t="inlineStr">
         <is>
           <t>АРМ.303411.004</t>
         </is>
       </c>
-      <c r="G4" s="3" t="n"/>
-      <c r="H4" s="3" t="inlineStr">
+      <c r="H4" s="3" t="n"/>
+      <c r="I4" s="3" t="inlineStr">
         <is>
           <t>Спецификации/АРМ.303411.000 Редуктор колёсный.pdf</t>
         </is>
       </c>
-      <c r="I4" s="3" t="inlineStr">
+      <c r="J4" s="3" t="inlineStr">
         <is>
           <t>Спецификации/АРМ.303411.000 Редуктор колёсный.pdf, стр. 1</t>
         </is>
@@ -930,31 +951,36 @@
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
+          <t>B1.ORPHAN.001</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
           <t>Средняя</t>
         </is>
       </c>
-      <c r="D5" s="3" t="inlineStr">
+      <c r="E5" s="3" t="inlineStr">
         <is>
           <t>АРМ.303412.007</t>
         </is>
       </c>
-      <c r="E5" s="3" t="inlineStr">
+      <c r="F5" s="3" t="inlineStr">
         <is>
           <t>Документ АРМ.303412.007 «Кронштейн» (Чертежи/АРМ.303412.007 Кронштейн.pdf) есть в комплекте, но не указан ни в одной спецификации</t>
         </is>
       </c>
-      <c r="F5" s="3" t="n"/>
-      <c r="G5" s="3" t="inlineStr">
+      <c r="G5" s="3" t="n"/>
+      <c r="H5" s="3" t="inlineStr">
         <is>
           <t>Чертежи/АРМ.303412.007 Кронштейн.pdf</t>
         </is>
       </c>
-      <c r="H5" s="3" t="inlineStr">
+      <c r="I5" s="3" t="inlineStr">
         <is>
           <t>Чертежи/АРМ.303412.007 Кронштейн.pdf</t>
         </is>
       </c>
-      <c r="I5" s="3" t="inlineStr">
+      <c r="J5" s="3" t="inlineStr">
         <is>
           <t>Чертежи/АРМ.303412.007 Кронштейн.pdf, стр. 1</t>
         </is>
@@ -971,32 +997,37 @@
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
+          <t>B1.DUP.001</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
           <t>Высокая</t>
         </is>
       </c>
-      <c r="D6" s="3" t="inlineStr">
+      <c r="E6" s="3" t="inlineStr">
         <is>
           <t>АРМ.303411.201</t>
         </is>
       </c>
-      <c r="E6" s="3" t="inlineStr">
+      <c r="F6" s="3" t="inlineStr">
         <is>
           <t>Обозначение АРМ.303411.201 присвоено 2 документам: Чертежи/АРМ.303411.201 Вал ведомый.pdf, Чертежи/Вал_изм3.pdf</t>
         </is>
       </c>
-      <c r="F6" s="3" t="n"/>
-      <c r="G6" s="3" t="inlineStr">
+      <c r="G6" s="3" t="n"/>
+      <c r="H6" s="3" t="inlineStr">
         <is>
           <t>Чертежи/АРМ.303411.201 Вал ведомый.pdf, Чертежи/Вал_изм3.pdf</t>
         </is>
       </c>
-      <c r="H6" s="3" t="inlineStr">
+      <c r="I6" s="3" t="inlineStr">
         <is>
           <t>Чертежи/Вал_изм3.pdf
 Чертежи/АРМ.303411.201 Вал ведомый.pdf</t>
         </is>
       </c>
-      <c r="I6" s="3" t="inlineStr">
+      <c r="J6" s="3" t="inlineStr">
         <is>
           <t>Чертежи/АРМ.303411.201 Вал ведомый.pdf, стр. 1
 Чертежи/Вал_изм3.pdf, стр. 1</t>
@@ -1014,32 +1045,37 @@
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
+          <t>B1.VERSION.001</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
           <t>Средняя</t>
         </is>
       </c>
-      <c r="D7" s="3" t="inlineStr">
+      <c r="E7" s="3" t="inlineStr">
         <is>
           <t>АРМ.303411.201</t>
         </is>
       </c>
-      <c r="E7" s="3" t="inlineStr">
+      <c r="F7" s="3" t="inlineStr">
         <is>
           <t>В комплекте несколько версий АРМ.303411.201 с разным номером изменения или литерой: Чертежи/АРМ.303411.201 Вал ведомый.pdf: изм. 2, лит. О1; Чертежи/Вал_изм3.pdf: изм. 3, лит. О1</t>
         </is>
       </c>
-      <c r="F7" s="3" t="n"/>
-      <c r="G7" s="3" t="inlineStr">
+      <c r="G7" s="3" t="n"/>
+      <c r="H7" s="3" t="inlineStr">
         <is>
           <t>Чертежи/АРМ.303411.201 Вал ведомый.pdf: изм. 2, лит. О1; Чертежи/Вал_изм3.pdf: изм. 3, лит. О1</t>
         </is>
       </c>
-      <c r="H7" s="3" t="inlineStr">
+      <c r="I7" s="3" t="inlineStr">
         <is>
           <t>Чертежи/Вал_изм3.pdf
 Чертежи/АРМ.303411.201 Вал ведомый.pdf</t>
         </is>
       </c>
-      <c r="I7" s="3" t="inlineStr">
+      <c r="J7" s="3" t="inlineStr">
         <is>
           <t>Чертежи/АРМ.303411.201 Вал ведомый.pdf, стр. 1
 Чертежи/Вал_изм3.pdf, стр. 1</t>
@@ -1057,35 +1093,40 @@
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
+          <t>B1.NAME.001</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
           <t>Средняя</t>
         </is>
       </c>
-      <c r="D8" s="3" t="inlineStr">
+      <c r="E8" s="3" t="inlineStr">
         <is>
           <t>АРМ.303411.002</t>
         </is>
       </c>
-      <c r="E8" s="3" t="inlineStr">
+      <c r="F8" s="3" t="inlineStr">
         <is>
           <t>АРМ.303411.002: в спецификации «Водило», на чертеже «Водило планетарное»</t>
         </is>
       </c>
-      <c r="F8" s="3" t="inlineStr">
+      <c r="G8" s="3" t="inlineStr">
         <is>
           <t>Водило</t>
         </is>
       </c>
-      <c r="G8" s="3" t="inlineStr">
+      <c r="H8" s="3" t="inlineStr">
         <is>
           <t>Водило планетарное</t>
         </is>
       </c>
-      <c r="H8" s="3" t="inlineStr">
+      <c r="I8" s="3" t="inlineStr">
         <is>
           <t>Чертежи/АРМ.303411.002 Водило.pdf</t>
         </is>
       </c>
-      <c r="I8" s="3" t="inlineStr">
+      <c r="J8" s="3" t="inlineStr">
         <is>
           <t>Чертежи/АРМ.303411.002 Водило.pdf, стр. 1</t>
         </is>
@@ -1102,36 +1143,41 @@
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
+          <t>B1.LITERA.001</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
           <t>Средняя</t>
         </is>
       </c>
-      <c r="D9" s="3" t="inlineStr">
+      <c r="E9" s="3" t="inlineStr">
         <is>
           <t>АРМ.303411.000</t>
         </is>
       </c>
-      <c r="E9" s="3" t="inlineStr">
+      <c r="F9" s="3" t="inlineStr">
         <is>
           <t>АРМ.303411.000: литера спецификации «О1», сборочного чертежа «О»</t>
         </is>
       </c>
-      <c r="F9" s="3" t="inlineStr">
+      <c r="G9" s="3" t="inlineStr">
         <is>
           <t>О1</t>
         </is>
       </c>
-      <c r="G9" s="3" t="inlineStr">
+      <c r="H9" s="3" t="inlineStr">
         <is>
           <t>О</t>
         </is>
       </c>
-      <c r="H9" s="3" t="inlineStr">
+      <c r="I9" s="3" t="inlineStr">
         <is>
           <t>Чертежи/АРМ.303411.000 СБ.pdf
 Спецификации/АРМ.303411.000 Редуктор колёсный.pdf</t>
         </is>
       </c>
-      <c r="I9" s="3" t="inlineStr">
+      <c r="J9" s="3" t="inlineStr">
         <is>
           <t>Спецификации/АРМ.303411.000 Редуктор колёсный.pdf, стр. 1
 Чертежи/АРМ.303411.000 СБ.pdf, стр. 1</t>
@@ -1149,36 +1195,41 @@
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
+          <t>B1.LITERA.002</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
           <t>Средняя</t>
         </is>
       </c>
-      <c r="D10" s="3" t="inlineStr">
+      <c r="E10" s="3" t="inlineStr">
         <is>
           <t>АРМ.303411.101</t>
         </is>
       </c>
-      <c r="E10" s="3" t="inlineStr">
+      <c r="F10" s="3" t="inlineStr">
         <is>
           <t>АРМ.303411.101: литера «О» ниже литеры сборочной единицы АРМ.303411.100 «О1»</t>
         </is>
       </c>
-      <c r="F10" s="3" t="inlineStr">
+      <c r="G10" s="3" t="inlineStr">
         <is>
           <t>не ниже О1</t>
         </is>
       </c>
-      <c r="G10" s="3" t="inlineStr">
+      <c r="H10" s="3" t="inlineStr">
         <is>
           <t>О</t>
         </is>
       </c>
-      <c r="H10" s="3" t="inlineStr">
+      <c r="I10" s="3" t="inlineStr">
         <is>
           <t>Спецификации/АРМ.303411.100 Корпус в сборе.pdf
 Чертежи/АРМ.303411.101 Корпус.pdf</t>
         </is>
       </c>
-      <c r="I10" s="3" t="inlineStr">
+      <c r="J10" s="3" t="inlineStr">
         <is>
           <t>Чертежи/АРМ.303411.101 Корпус.pdf, стр. 1
 Спецификации/АРМ.303411.100 Корпус в сборе.pdf, стр. 1</t>
@@ -1186,7 +1237,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I10"/>
+  <autoFilter ref="A1:J10"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
chore(frontend): rebuild the demo report on contract 1.3
The pages carry their sheet formats: the drawings are A3, the
specifications, the foreign act and the scan with its resolution are A4,
the unreadable scan has no format. Nothing else changed apart from the
settings hash and the times.
</commit_message>
<xml_diff>
--- a/frontend/public/demo/report.xlsx
+++ b/frontend/public/demo/report.xlsx
@@ -24,7 +24,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Параметры'!$A$1:$N$79</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Критичные параметры'!$A$1:$H$25</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Спецификации'!$A$1:$H$26</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Документы'!$A$1:$I$23</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Документы'!$A$1:$J$23</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Качество'!$A$1:$G$22</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -484,7 +484,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-10-22T03:20:19+00:00</t>
+          <t>2026-10-22T15:22:06+00:00</t>
         </is>
       </c>
     </row>
@@ -520,7 +520,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>63cd3acc4802cb6cb498201bf52b75da245da18316a4711d03f7e8b57b9a47bc</t>
+          <t>9b244b4c1dc798954865f1f2ecd042c4545d79e5c7c218230ce954bdfffd4a30</t>
         </is>
       </c>
     </row>
@@ -9372,18 +9372,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I23"/>
+  <dimension ref="A1:J23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
     <col width="13" customWidth="1" min="3" max="3"/>
     <col width="6" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
-    <col width="28" customWidth="1" min="6" max="6"/>
-    <col width="20" customWidth="1" min="7" max="7"/>
-    <col width="50" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="28" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="8" max="8"/>
     <col width="50" customWidth="1" min="9" max="9"/>
+    <col width="50" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -9409,25 +9410,30 @@
       </c>
       <c r="E1" s="2" t="inlineStr">
         <is>
+          <t>Формат</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
           <t>Обозначение</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="G1" s="2" t="inlineStr">
         <is>
           <t>Наименование</t>
         </is>
       </c>
-      <c r="G1" s="2" t="inlineStr">
+      <c r="H1" s="2" t="inlineStr">
         <is>
           <t>Статус</t>
         </is>
       </c>
-      <c r="H1" s="2" t="inlineStr">
+      <c r="I1" s="2" t="inlineStr">
         <is>
           <t>Проблема</t>
         </is>
       </c>
-      <c r="I1" s="2" t="inlineStr">
+      <c r="J1" s="2" t="inlineStr">
         <is>
           <t>Примечания</t>
         </is>
@@ -9454,17 +9460,18 @@
       </c>
       <c r="E2" s="3" t="n"/>
       <c r="F2" s="3" t="n"/>
-      <c r="G2" s="3" t="inlineStr">
+      <c r="G2" s="3" t="n"/>
+      <c r="H2" s="3" t="inlineStr">
         <is>
           <t>Неподдерживаемый формат</t>
         </is>
       </c>
-      <c r="H2" s="3" t="inlineStr">
+      <c r="I2" s="3" t="inlineStr">
         <is>
           <t>Формат файла не поддерживается (.db): ожидаются PDF или изображения</t>
         </is>
       </c>
-      <c r="I2" s="3" t="inlineStr"/>
+      <c r="J2" s="3" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
@@ -9485,19 +9492,24 @@
       <c r="D3" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="E3" s="3" t="n"/>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>A4</t>
+        </is>
+      </c>
       <c r="F3" s="3" t="n"/>
-      <c r="G3" s="3" t="inlineStr">
+      <c r="G3" s="3" t="n"/>
+      <c r="H3" s="3" t="inlineStr">
         <is>
           <t>Посторонний документ</t>
         </is>
       </c>
-      <c r="H3" s="3" t="inlineStr">
+      <c r="I3" s="3" t="inlineStr">
         <is>
           <t>Посторонний документ: нет основной надписи чертежа и граф спецификации</t>
         </is>
       </c>
-      <c r="I3" s="3" t="inlineStr"/>
+      <c r="J3" s="3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
@@ -9520,21 +9532,26 @@
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
+          <t>A4</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
           <t>АРМ.303411.000</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="G4" s="3" t="inlineStr">
         <is>
           <t>Редуктор колёсный</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="H4" s="3" t="inlineStr">
         <is>
           <t>Обработан</t>
         </is>
       </c>
-      <c r="H4" s="3" t="n"/>
-      <c r="I4" s="3" t="inlineStr"/>
+      <c r="I4" s="3" t="n"/>
+      <c r="J4" s="3" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -9557,21 +9574,26 @@
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
+          <t>A4</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
           <t>АРМ.303411.100</t>
         </is>
       </c>
-      <c r="F5" s="3" t="inlineStr">
+      <c r="G5" s="3" t="inlineStr">
         <is>
           <t>Корпус в сборе</t>
         </is>
       </c>
-      <c r="G5" s="3" t="inlineStr">
+      <c r="H5" s="3" t="inlineStr">
         <is>
           <t>Обработан</t>
         </is>
       </c>
-      <c r="H5" s="3" t="n"/>
-      <c r="I5" s="3" t="inlineStr"/>
+      <c r="I5" s="3" t="n"/>
+      <c r="J5" s="3" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
@@ -9594,21 +9616,26 @@
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
+          <t>A4</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
           <t>АРМ.303411.200</t>
         </is>
       </c>
-      <c r="F6" s="3" t="inlineStr">
+      <c r="G6" s="3" t="inlineStr">
         <is>
           <t>Вал ведомый в сборе</t>
         </is>
       </c>
-      <c r="G6" s="3" t="inlineStr">
+      <c r="H6" s="3" t="inlineStr">
         <is>
           <t>Обработан</t>
         </is>
       </c>
-      <c r="H6" s="3" t="n"/>
-      <c r="I6" s="3" t="inlineStr"/>
+      <c r="I6" s="3" t="n"/>
+      <c r="J6" s="3" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
@@ -9631,21 +9658,26 @@
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
+          <t>A3</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
           <t>АРМ.303411.000 СБ</t>
         </is>
       </c>
-      <c r="F7" s="3" t="inlineStr">
+      <c r="G7" s="3" t="inlineStr">
         <is>
           <t>Редуктор колёсный</t>
         </is>
       </c>
-      <c r="G7" s="3" t="inlineStr">
+      <c r="H7" s="3" t="inlineStr">
         <is>
           <t>Обработан</t>
         </is>
       </c>
-      <c r="H7" s="3" t="n"/>
-      <c r="I7" s="3" t="inlineStr"/>
+      <c r="I7" s="3" t="n"/>
+      <c r="J7" s="3" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
@@ -9668,21 +9700,26 @@
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
+          <t>A3</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
           <t>АРМ.303411.001</t>
         </is>
       </c>
-      <c r="F8" s="3" t="inlineStr">
+      <c r="G8" s="3" t="inlineStr">
         <is>
           <t>Шестерня солнечная</t>
         </is>
       </c>
-      <c r="G8" s="3" t="inlineStr">
+      <c r="H8" s="3" t="inlineStr">
         <is>
           <t>Обработан</t>
         </is>
       </c>
-      <c r="H8" s="3" t="n"/>
-      <c r="I8" s="3" t="inlineStr"/>
+      <c r="I8" s="3" t="n"/>
+      <c r="J8" s="3" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
@@ -9705,21 +9742,26 @@
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
+          <t>A3</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
           <t>АРМ.303411.002</t>
         </is>
       </c>
-      <c r="F9" s="3" t="inlineStr">
+      <c r="G9" s="3" t="inlineStr">
         <is>
           <t>Водило планетарное</t>
         </is>
       </c>
-      <c r="G9" s="3" t="inlineStr">
+      <c r="H9" s="3" t="inlineStr">
         <is>
           <t>Обработан</t>
         </is>
       </c>
-      <c r="H9" s="3" t="n"/>
-      <c r="I9" s="3" t="inlineStr"/>
+      <c r="I9" s="3" t="n"/>
+      <c r="J9" s="3" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
@@ -9742,21 +9784,26 @@
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
+          <t>A4</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
           <t>АРМ.303411.003</t>
         </is>
       </c>
-      <c r="F10" s="3" t="inlineStr">
+      <c r="G10" s="3" t="inlineStr">
         <is>
           <t>Крышка торцевая</t>
         </is>
       </c>
-      <c r="G10" s="3" t="inlineStr">
+      <c r="H10" s="3" t="inlineStr">
         <is>
           <t>Обработан</t>
         </is>
       </c>
-      <c r="H10" s="3" t="n"/>
-      <c r="I10" s="3" t="inlineStr">
+      <c r="I10" s="3" t="n"/>
+      <c r="J10" s="3" t="inlineStr">
         <is>
           <t>Текст получен распознаванием скана (OCR) — значения требуют проверки</t>
         </is>
@@ -9783,21 +9830,26 @@
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
+          <t>A4</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
           <t>АРМ.303411.005</t>
         </is>
       </c>
-      <c r="F11" s="3" t="inlineStr">
+      <c r="G11" s="3" t="inlineStr">
         <is>
           <t>Гайка специальная</t>
         </is>
       </c>
-      <c r="G11" s="3" t="inlineStr">
+      <c r="H11" s="3" t="inlineStr">
         <is>
           <t>Обработан</t>
         </is>
       </c>
-      <c r="H11" s="3" t="n"/>
-      <c r="I11" s="3" t="inlineStr"/>
+      <c r="I11" s="3" t="n"/>
+      <c r="J11" s="3" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
@@ -9820,21 +9872,26 @@
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
+          <t>A3</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
           <t>АРМ.303411.100 СБ</t>
         </is>
       </c>
-      <c r="F12" s="3" t="inlineStr">
+      <c r="G12" s="3" t="inlineStr">
         <is>
           <t>Корпус в сборе</t>
         </is>
       </c>
-      <c r="G12" s="3" t="inlineStr">
+      <c r="H12" s="3" t="inlineStr">
         <is>
           <t>Обработан</t>
         </is>
       </c>
-      <c r="H12" s="3" t="n"/>
-      <c r="I12" s="3" t="inlineStr"/>
+      <c r="I12" s="3" t="n"/>
+      <c r="J12" s="3" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
@@ -9857,21 +9914,26 @@
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
+          <t>A3</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
           <t>АРМ.303411.101</t>
         </is>
       </c>
-      <c r="F13" s="3" t="inlineStr">
+      <c r="G13" s="3" t="inlineStr">
         <is>
           <t>Корпус</t>
         </is>
       </c>
-      <c r="G13" s="3" t="inlineStr">
+      <c r="H13" s="3" t="inlineStr">
         <is>
           <t>Обработан</t>
         </is>
       </c>
-      <c r="H13" s="3" t="n"/>
-      <c r="I13" s="3" t="inlineStr"/>
+      <c r="I13" s="3" t="n"/>
+      <c r="J13" s="3" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
@@ -9894,21 +9956,26 @@
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
+          <t>A3</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
           <t>АРМ.303411.102</t>
         </is>
       </c>
-      <c r="F14" s="3" t="inlineStr">
+      <c r="G14" s="3" t="inlineStr">
         <is>
           <t>Крышка</t>
         </is>
       </c>
-      <c r="G14" s="3" t="inlineStr">
+      <c r="H14" s="3" t="inlineStr">
         <is>
           <t>Обработан</t>
         </is>
       </c>
-      <c r="H14" s="3" t="n"/>
-      <c r="I14" s="3" t="inlineStr"/>
+      <c r="I14" s="3" t="n"/>
+      <c r="J14" s="3" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
@@ -9931,21 +9998,26 @@
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
+          <t>A3</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
           <t>АРМ.303411.200 СБ</t>
         </is>
       </c>
-      <c r="F15" s="3" t="inlineStr">
+      <c r="G15" s="3" t="inlineStr">
         <is>
           <t>Вал ведомый в сборе</t>
         </is>
       </c>
-      <c r="G15" s="3" t="inlineStr">
+      <c r="H15" s="3" t="inlineStr">
         <is>
           <t>Обработан</t>
         </is>
       </c>
-      <c r="H15" s="3" t="n"/>
-      <c r="I15" s="3" t="inlineStr"/>
+      <c r="I15" s="3" t="n"/>
+      <c r="J15" s="3" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
@@ -9968,21 +10040,26 @@
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
+          <t>A3</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
           <t>АРМ.303411.201</t>
         </is>
       </c>
-      <c r="F16" s="3" t="inlineStr">
+      <c r="G16" s="3" t="inlineStr">
         <is>
           <t>Вал ведомый</t>
         </is>
       </c>
-      <c r="G16" s="3" t="inlineStr">
+      <c r="H16" s="3" t="inlineStr">
         <is>
           <t>Обработан</t>
         </is>
       </c>
-      <c r="H16" s="3" t="n"/>
-      <c r="I16" s="3" t="inlineStr"/>
+      <c r="I16" s="3" t="n"/>
+      <c r="J16" s="3" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
@@ -10005,21 +10082,26 @@
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
+          <t>A3</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
           <t>АРМ.303411.202</t>
         </is>
       </c>
-      <c r="F17" s="3" t="inlineStr">
+      <c r="G17" s="3" t="inlineStr">
         <is>
           <t>Колесо зубчатое</t>
         </is>
       </c>
-      <c r="G17" s="3" t="inlineStr">
+      <c r="H17" s="3" t="inlineStr">
         <is>
           <t>Обработан</t>
         </is>
       </c>
-      <c r="H17" s="3" t="n"/>
-      <c r="I17" s="3" t="inlineStr"/>
+      <c r="I17" s="3" t="n"/>
+      <c r="J17" s="3" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
@@ -10042,21 +10124,26 @@
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
+          <t>A4</t>
+        </is>
+      </c>
+      <c r="F18" s="3" t="inlineStr">
+        <is>
           <t>АРМ.303411.203</t>
         </is>
       </c>
-      <c r="F18" s="3" t="inlineStr">
+      <c r="G18" s="3" t="inlineStr">
         <is>
           <t>Кольцо распорное</t>
         </is>
       </c>
-      <c r="G18" s="3" t="inlineStr">
+      <c r="H18" s="3" t="inlineStr">
         <is>
           <t>Обработан</t>
         </is>
       </c>
-      <c r="H18" s="3" t="n"/>
-      <c r="I18" s="3" t="inlineStr">
+      <c r="I18" s="3" t="n"/>
+      <c r="J18" s="3" t="inlineStr">
         <is>
           <t>Текст получен распознаванием скана (OCR) — значения требуют проверки</t>
         </is>
@@ -10083,21 +10170,26 @@
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
+          <t>A4</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
           <t>АРМ.303411.300 СБ</t>
         </is>
       </c>
-      <c r="F19" s="3" t="inlineStr">
+      <c r="G19" s="3" t="inlineStr">
         <is>
           <t>Сателлит в сборе</t>
         </is>
       </c>
-      <c r="G19" s="3" t="inlineStr">
+      <c r="H19" s="3" t="inlineStr">
         <is>
           <t>Обработан</t>
         </is>
       </c>
-      <c r="H19" s="3" t="n"/>
-      <c r="I19" s="3" t="inlineStr"/>
+      <c r="I19" s="3" t="n"/>
+      <c r="J19" s="3" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
@@ -10120,21 +10212,26 @@
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
+          <t>A3</t>
+        </is>
+      </c>
+      <c r="F20" s="3" t="inlineStr">
+        <is>
           <t>АРМ.303412.007</t>
         </is>
       </c>
-      <c r="F20" s="3" t="inlineStr">
+      <c r="G20" s="3" t="inlineStr">
         <is>
           <t>Кронштейн</t>
         </is>
       </c>
-      <c r="G20" s="3" t="inlineStr">
+      <c r="H20" s="3" t="inlineStr">
         <is>
           <t>Обработан</t>
         </is>
       </c>
-      <c r="H20" s="3" t="n"/>
-      <c r="I20" s="3" t="inlineStr"/>
+      <c r="I20" s="3" t="n"/>
+      <c r="J20" s="3" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
@@ -10157,21 +10254,26 @@
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
+          <t>A3</t>
+        </is>
+      </c>
+      <c r="F21" s="3" t="inlineStr">
+        <is>
           <t>АРМ.303411.201</t>
         </is>
       </c>
-      <c r="F21" s="3" t="inlineStr">
+      <c r="G21" s="3" t="inlineStr">
         <is>
           <t>Вал ведомый</t>
         </is>
       </c>
-      <c r="G21" s="3" t="inlineStr">
+      <c r="H21" s="3" t="inlineStr">
         <is>
           <t>Обработан</t>
         </is>
       </c>
-      <c r="H21" s="3" t="n"/>
-      <c r="I21" s="3" t="inlineStr"/>
+      <c r="I21" s="3" t="n"/>
+      <c r="J21" s="3" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
@@ -10194,17 +10296,18 @@
       </c>
       <c r="E22" s="3" t="n"/>
       <c r="F22" s="3" t="n"/>
-      <c r="G22" s="3" t="inlineStr">
+      <c r="G22" s="3" t="n"/>
+      <c r="H22" s="3" t="inlineStr">
         <is>
           <t>Повреждён</t>
         </is>
       </c>
-      <c r="H22" s="3" t="inlineStr">
+      <c r="I22" s="3" t="inlineStr">
         <is>
           <t>Файл повреждён или не открывается: Failed to load document (PDFium: Data format error).</t>
         </is>
       </c>
-      <c r="I22" s="3" t="inlineStr"/>
+      <c r="J22" s="3" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
@@ -10227,20 +10330,21 @@
       </c>
       <c r="E23" s="3" t="n"/>
       <c r="F23" s="3" t="n"/>
-      <c r="G23" s="3" t="inlineStr">
+      <c r="G23" s="3" t="n"/>
+      <c r="H23" s="3" t="inlineStr">
         <is>
           <t>Нечитаемый скан</t>
         </is>
       </c>
-      <c r="H23" s="3" t="inlineStr">
+      <c r="I23" s="3" t="inlineStr">
         <is>
           <t>Нечитаемый скан: низкий контраст изображения</t>
         </is>
       </c>
-      <c r="I23" s="3" t="inlineStr"/>
+      <c r="J23" s="3" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I23"/>
+  <autoFilter ref="A1:J23"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
eval: re-measure on the GOST lettering, OCR misreads it more often
With the demo kit in OpenGost Type A, Tesseract reads the title blocks of
the scans right in 0.375 of the fields instead of 0.625, and one OCR
misread of a name on a scan adds a false name mismatch. Block 1 with OCR on
the 20 synthetic kits: recall 0.835 instead of 0.861, precision 0.537
instead of 0.63; without OCR the numbers stay. The demo report of the web
UI is rebuilt from the new kit. README and the plan give the new numbers.
</commit_message>
<xml_diff>
--- a/frontend/public/demo/report.xlsx
+++ b/frontend/public/demo/report.xlsx
@@ -18,11 +18,11 @@
     <sheet name="Качество" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Расхождения'!$A$1:$J$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Расхождения'!$A$1:$J$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Дерево изделия'!$A$1:$J$27</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Основные надписи'!$A$1:$L$16</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Параметры'!$A$1:$N$79</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Критичные параметры'!$A$1:$H$25</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Параметры'!$A$1:$N$77</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Критичные параметры'!$A$1:$H$24</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Спецификации'!$A$1:$H$26</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Документы'!$A$1:$J$23</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Качество'!$A$1:$G$22</definedName>
@@ -484,7 +484,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-10-22T15:22:06+00:00</t>
+          <t>2026-10-26T09:41:18+00:00</t>
         </is>
       </c>
     </row>
@@ -583,7 +583,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="13">
@@ -593,7 +593,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="14">
@@ -634,7 +634,7 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="19">
@@ -739,7 +739,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J10"/>
+  <dimension ref="A1:J11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1138,12 +1138,12 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>Расхождение литеры / изменения</t>
+          <t>Расхождение наименования</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>B1.LITERA.001</t>
+          <t>B1.NAME.001</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
@@ -1153,34 +1153,32 @@
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>АРМ.303411.000</t>
+          <t>АРМ.303411.003</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>АРМ.303411.000: литера спецификации «О1», сборочного чертежа «О»</t>
+          <t>АРМ.303411.003: в спецификации «Крышка торцевая», на чертеже «Крышка торцебоя»</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
         <is>
-          <t>О1</t>
+          <t>Крышка торцевая</t>
         </is>
       </c>
       <c r="H9" s="3" t="inlineStr">
         <is>
-          <t>О</t>
+          <t>Крышка торцебоя</t>
         </is>
       </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>Чертежи/АРМ.303411.000 СБ.pdf
-Спецификации/АРМ.303411.000 Редуктор колёсный.pdf</t>
+          <t>Чертежи/АРМ.303411.003 Крышка торцевая.pdf</t>
         </is>
       </c>
       <c r="J9" s="3" t="inlineStr">
         <is>
-          <t>Спецификации/АРМ.303411.000 Редуктор колёсный.pdf, стр. 1
-Чертежи/АРМ.303411.000 СБ.pdf, стр. 1</t>
+          <t>Чертежи/АРМ.303411.003 Крышка торцевая.pdf, стр. 1</t>
         </is>
       </c>
     </row>
@@ -1195,41 +1193,93 @@
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
+          <t>B1.LITERA.001</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>Средняя</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>АРМ.303411.000</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>АРМ.303411.000: литера спецификации «О1», сборочного чертежа «О»</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="inlineStr">
+        <is>
+          <t>О1</t>
+        </is>
+      </c>
+      <c r="H10" s="3" t="inlineStr">
+        <is>
+          <t>О</t>
+        </is>
+      </c>
+      <c r="I10" s="3" t="inlineStr">
+        <is>
+          <t>Чертежи/АРМ.303411.000 СБ.pdf
+Спецификации/АРМ.303411.000 Редуктор колёсный.pdf</t>
+        </is>
+      </c>
+      <c r="J10" s="3" t="inlineStr">
+        <is>
+          <t>Спецификации/АРМ.303411.000 Редуктор колёсный.pdf, стр. 1
+Чертежи/АРМ.303411.000 СБ.pdf, стр. 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>Расхождение литеры / изменения</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
           <t>B1.LITERA.002</t>
         </is>
       </c>
-      <c r="D10" s="3" t="inlineStr">
+      <c r="D11" s="3" t="inlineStr">
         <is>
           <t>Средняя</t>
         </is>
       </c>
-      <c r="E10" s="3" t="inlineStr">
+      <c r="E11" s="3" t="inlineStr">
         <is>
           <t>АРМ.303411.101</t>
         </is>
       </c>
-      <c r="F10" s="3" t="inlineStr">
+      <c r="F11" s="3" t="inlineStr">
         <is>
           <t>АРМ.303411.101: литера «О» ниже литеры сборочной единицы АРМ.303411.100 «О1»</t>
         </is>
       </c>
-      <c r="G10" s="3" t="inlineStr">
+      <c r="G11" s="3" t="inlineStr">
         <is>
           <t>не ниже О1</t>
         </is>
       </c>
-      <c r="H10" s="3" t="inlineStr">
+      <c r="H11" s="3" t="inlineStr">
         <is>
           <t>О</t>
         </is>
       </c>
-      <c r="I10" s="3" t="inlineStr">
+      <c r="I11" s="3" t="inlineStr">
         <is>
           <t>Спецификации/АРМ.303411.100 Корпус в сборе.pdf
 Чертежи/АРМ.303411.101 Корпус.pdf</t>
         </is>
       </c>
-      <c r="J10" s="3" t="inlineStr">
+      <c r="J11" s="3" t="inlineStr">
         <is>
           <t>Чертежи/АРМ.303411.101 Корпус.pdf, стр. 1
 Спецификации/АРМ.303411.100 Корпус в сборе.pdf, стр. 1</t>
@@ -1237,7 +1287,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J10"/>
+  <autoFilter ref="A1:J11"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2171,7 +2221,7 @@
       </c>
       <c r="I21" s="3" t="inlineStr">
         <is>
-          <t>Есть</t>
+          <t>Есть замечания</t>
         </is>
       </c>
       <c r="J21" s="3" t="inlineStr">
@@ -2698,20 +2748,16 @@
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>Крышка торцевая</t>
+          <t>Крышка торцебоя</t>
         </is>
       </c>
       <c r="D5" s="3" t="n"/>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>1,2</t>
-        </is>
-      </c>
-      <c r="F5" s="3" t="inlineStr">
-        <is>
-          <t>1:1</t>
-        </is>
-      </c>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="n"/>
       <c r="G5" s="3" t="inlineStr">
         <is>
           <t>О1</t>
@@ -3121,11 +3167,7 @@
           <t>0,22</t>
         </is>
       </c>
-      <c r="F13" s="3" t="inlineStr">
-        <is>
-          <t>1:1</t>
-        </is>
-      </c>
+      <c r="F13" s="3" t="n"/>
       <c r="G13" s="3" t="inlineStr">
         <is>
           <t>О1</t>
@@ -3309,7 +3351,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N79"/>
+  <dimension ref="A1:N77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -4302,38 +4344,40 @@
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>Крышка торцевая</t>
+          <t>Крышка торцебоя</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>Покрытие</t>
+          <t>Шероховатость</t>
         </is>
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>Хим.Окс.прм</t>
-        </is>
-      </c>
-      <c r="E19" s="3" t="n"/>
+          <t>Ra 3,2</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="n">
+        <v>3.2</v>
+      </c>
       <c r="F19" s="3" t="n"/>
       <c r="G19" s="3" t="n"/>
-      <c r="H19" s="3" t="n"/>
+      <c r="H19" s="3" t="inlineStr">
+        <is>
+          <t>мкм</t>
+        </is>
+      </c>
       <c r="I19" s="3" t="inlineStr">
         <is>
-          <t>Хим.Окс.прм</t>
+          <t>Ra</t>
         </is>
       </c>
       <c r="J19" s="3" t="n"/>
       <c r="K19" s="3" t="inlineStr"/>
-      <c r="L19" s="3" t="inlineStr">
-        <is>
-          <t>да</t>
-        </is>
-      </c>
+      <c r="L19" s="3" t="inlineStr"/>
       <c r="M19" s="3" t="inlineStr">
         <is>
-          <t>. Покрытие Хим.Окс.прм.</t>
+          <t>Ra 3,2</t>
         </is>
       </c>
       <c r="N19" s="3" t="inlineStr">
@@ -4345,94 +4389,100 @@
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t>АРМ.303411.003</t>
+          <t>АРМ.303411.005</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>Крышка торцевая</t>
+          <t>Гайка специальная</t>
         </is>
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>Общие допуски</t>
+          <t>Твёрдость</t>
         </is>
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>Неуказанные отклонения</t>
+          <t>Твёрдость HRC</t>
         </is>
       </c>
       <c r="E20" s="3" t="n"/>
-      <c r="F20" s="3" t="n"/>
-      <c r="G20" s="3" t="n"/>
-      <c r="H20" s="3" t="n"/>
-      <c r="I20" s="3" t="n"/>
+      <c r="F20" s="3" t="n">
+        <v>30</v>
+      </c>
+      <c r="G20" s="3" t="n">
+        <v>35</v>
+      </c>
+      <c r="H20" s="3" t="inlineStr">
+        <is>
+          <t>HRC</t>
+        </is>
+      </c>
+      <c r="I20" s="3" t="inlineStr">
+        <is>
+          <t>HRC</t>
+        </is>
+      </c>
       <c r="J20" s="3" t="n"/>
-      <c r="K20" s="3" t="inlineStr">
-        <is>
-          <t>да</t>
-        </is>
-      </c>
+      <c r="K20" s="3" t="inlineStr"/>
       <c r="L20" s="3" t="inlineStr"/>
       <c r="M20" s="3" t="inlineStr">
         <is>
-          <t>Неуказанные предельные отклонения размеров: Н14, 114, +1T14/2.</t>
+          <t>30...35 HRC.</t>
         </is>
       </c>
       <c r="N20" s="3" t="inlineStr">
         <is>
-          <t>Чертежи/АРМ.303411.003 Крышка торцевая.pdf, стр. 1</t>
+          <t>Чертежи/АРМ.303411.005 Гайка специальная.pdf, стр. 1</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>АРМ.303411.003</t>
+          <t>АРМ.303411.005</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>Крышка торцевая</t>
+          <t>Гайка специальная</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>Шероховатость</t>
+          <t>Покрытие</t>
         </is>
       </c>
       <c r="D21" s="3" t="inlineStr">
         <is>
-          <t>Ra 3,2</t>
-        </is>
-      </c>
-      <c r="E21" s="3" t="n">
-        <v>3.2</v>
-      </c>
+          <t>Ц9.хр</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="n"/>
       <c r="F21" s="3" t="n"/>
       <c r="G21" s="3" t="n"/>
-      <c r="H21" s="3" t="inlineStr">
-        <is>
-          <t>мкм</t>
-        </is>
-      </c>
+      <c r="H21" s="3" t="n"/>
       <c r="I21" s="3" t="inlineStr">
         <is>
-          <t>Ra</t>
+          <t>Ц9.хр</t>
         </is>
       </c>
       <c r="J21" s="3" t="n"/>
       <c r="K21" s="3" t="inlineStr"/>
-      <c r="L21" s="3" t="inlineStr"/>
+      <c r="L21" s="3" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
       <c r="M21" s="3" t="inlineStr">
         <is>
-          <t>Ва 3,2</t>
+          <t>Покрытие Ц9.хр.</t>
         </is>
       </c>
       <c r="N21" s="3" t="inlineStr">
         <is>
-          <t>Чертежи/АРМ.303411.003 Крышка торцевая.pdf, стр. 1</t>
+          <t>Чертежи/АРМ.303411.005 Гайка специальная.pdf, стр. 1</t>
         </is>
       </c>
     </row>
@@ -4449,37 +4499,35 @@
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>Твёрдость</t>
+          <t>Общие допуски</t>
         </is>
       </c>
       <c r="D22" s="3" t="inlineStr">
         <is>
-          <t>Твёрдость HRC</t>
+          <t>IT14</t>
         </is>
       </c>
       <c r="E22" s="3" t="n"/>
-      <c r="F22" s="3" t="n">
-        <v>30</v>
-      </c>
-      <c r="G22" s="3" t="n">
-        <v>35</v>
-      </c>
-      <c r="H22" s="3" t="inlineStr">
-        <is>
-          <t>HRC</t>
-        </is>
-      </c>
+      <c r="F22" s="3" t="n"/>
+      <c r="G22" s="3" t="n"/>
+      <c r="H22" s="3" t="n"/>
       <c r="I22" s="3" t="inlineStr">
         <is>
-          <t>HRC</t>
-        </is>
-      </c>
-      <c r="J22" s="3" t="n"/>
-      <c r="K22" s="3" t="inlineStr"/>
+          <t>H14, h14</t>
+        </is>
+      </c>
+      <c r="J22" s="3" t="n">
+        <v>14</v>
+      </c>
+      <c r="K22" s="3" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
       <c r="L22" s="3" t="inlineStr"/>
       <c r="M22" s="3" t="inlineStr">
         <is>
-          <t>30...35 HRC.</t>
+          <t>Неуказанные предельные отклонения размеров: H14, h14, ±IT14/2.</t>
         </is>
       </c>
       <c r="N22" s="3" t="inlineStr">
@@ -4501,33 +4549,35 @@
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>Покрытие</t>
+          <t>Допуск размера</t>
         </is>
       </c>
       <c r="D23" s="3" t="inlineStr">
         <is>
-          <t>Ц9.хр</t>
-        </is>
-      </c>
-      <c r="E23" s="3" t="n"/>
+          <t>М48×1,5-6H</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="n">
+        <v>48</v>
+      </c>
       <c r="F23" s="3" t="n"/>
       <c r="G23" s="3" t="n"/>
-      <c r="H23" s="3" t="n"/>
+      <c r="H23" s="3" t="inlineStr">
+        <is>
+          <t>мм</t>
+        </is>
+      </c>
       <c r="I23" s="3" t="inlineStr">
         <is>
-          <t>Ц9.хр</t>
+          <t>6H</t>
         </is>
       </c>
       <c r="J23" s="3" t="n"/>
       <c r="K23" s="3" t="inlineStr"/>
-      <c r="L23" s="3" t="inlineStr">
-        <is>
-          <t>да</t>
-        </is>
-      </c>
+      <c r="L23" s="3" t="inlineStr"/>
       <c r="M23" s="3" t="inlineStr">
         <is>
-          <t>Покрытие Ц9.хр.</t>
+          <t>М48×1,5-6H</t>
         </is>
       </c>
       <c r="N23" s="3" t="inlineStr">
@@ -4549,35 +4599,35 @@
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>Общие допуски</t>
+          <t>Шероховатость</t>
         </is>
       </c>
       <c r="D24" s="3" t="inlineStr">
         <is>
-          <t>IT14</t>
-        </is>
-      </c>
-      <c r="E24" s="3" t="n"/>
+          <t>Ra 3,2</t>
+        </is>
+      </c>
+      <c r="E24" s="3" t="n">
+        <v>3.2</v>
+      </c>
       <c r="F24" s="3" t="n"/>
       <c r="G24" s="3" t="n"/>
-      <c r="H24" s="3" t="n"/>
+      <c r="H24" s="3" t="inlineStr">
+        <is>
+          <t>мкм</t>
+        </is>
+      </c>
       <c r="I24" s="3" t="inlineStr">
         <is>
-          <t>H14, h14</t>
-        </is>
-      </c>
-      <c r="J24" s="3" t="n">
-        <v>14</v>
-      </c>
-      <c r="K24" s="3" t="inlineStr">
-        <is>
-          <t>да</t>
-        </is>
-      </c>
+          <t>Ra</t>
+        </is>
+      </c>
+      <c r="J24" s="3" t="n"/>
+      <c r="K24" s="3" t="inlineStr"/>
       <c r="L24" s="3" t="inlineStr"/>
       <c r="M24" s="3" t="inlineStr">
         <is>
-          <t>Неуказанные предельные отклонения размеров: H14, h14, ±IT14/2.</t>
+          <t>Ra 3,2</t>
         </is>
       </c>
       <c r="N24" s="3" t="inlineStr">
@@ -4599,35 +4649,39 @@
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>Допуск размера</t>
+          <t>Шероховатость</t>
         </is>
       </c>
       <c r="D25" s="3" t="inlineStr">
         <is>
-          <t>М48×1,5-6H</t>
+          <t>Ra 12,5</t>
         </is>
       </c>
       <c r="E25" s="3" t="n">
-        <v>48</v>
+        <v>12.5</v>
       </c>
       <c r="F25" s="3" t="n"/>
       <c r="G25" s="3" t="n"/>
       <c r="H25" s="3" t="inlineStr">
         <is>
-          <t>мм</t>
+          <t>мкм</t>
         </is>
       </c>
       <c r="I25" s="3" t="inlineStr">
         <is>
-          <t>6H</t>
+          <t>Ra</t>
         </is>
       </c>
       <c r="J25" s="3" t="n"/>
-      <c r="K25" s="3" t="inlineStr"/>
+      <c r="K25" s="3" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
       <c r="L25" s="3" t="inlineStr"/>
       <c r="M25" s="3" t="inlineStr">
         <is>
-          <t>М48×1,5-6H</t>
+          <t>√Ra 12,5 (√)</t>
         </is>
       </c>
       <c r="N25" s="3" t="inlineStr">
@@ -4639,104 +4693,94 @@
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
         <is>
-          <t>АРМ.303411.005</t>
+          <t>АРМ.303411.101</t>
         </is>
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>Гайка специальная</t>
+          <t>Корпус</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>Шероховатость</t>
+          <t>Общие допуски</t>
         </is>
       </c>
       <c r="D26" s="3" t="inlineStr">
         <is>
-          <t>Ra 3,2</t>
-        </is>
-      </c>
-      <c r="E26" s="3" t="n">
-        <v>3.2</v>
-      </c>
+          <t>IT14</t>
+        </is>
+      </c>
+      <c r="E26" s="3" t="n"/>
       <c r="F26" s="3" t="n"/>
       <c r="G26" s="3" t="n"/>
-      <c r="H26" s="3" t="inlineStr">
-        <is>
-          <t>мкм</t>
-        </is>
-      </c>
+      <c r="H26" s="3" t="n"/>
       <c r="I26" s="3" t="inlineStr">
         <is>
-          <t>Ra</t>
-        </is>
-      </c>
-      <c r="J26" s="3" t="n"/>
-      <c r="K26" s="3" t="inlineStr"/>
+          <t>H14, h14</t>
+        </is>
+      </c>
+      <c r="J26" s="3" t="n">
+        <v>14</v>
+      </c>
+      <c r="K26" s="3" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
       <c r="L26" s="3" t="inlineStr"/>
       <c r="M26" s="3" t="inlineStr">
         <is>
-          <t>Ra 3,2</t>
+          <t>Неуказанные предельные отклонения размеров: H14, h14, ±IT14/2.</t>
         </is>
       </c>
       <c r="N26" s="3" t="inlineStr">
         <is>
-          <t>Чертежи/АРМ.303411.005 Гайка специальная.pdf, стр. 1</t>
+          <t>Чертежи/АРМ.303411.101 Корпус.pdf, стр. 1</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
         <is>
-          <t>АРМ.303411.005</t>
+          <t>АРМ.303411.101</t>
         </is>
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>Гайка специальная</t>
+          <t>Корпус</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>Шероховатость</t>
+          <t>Покрытие</t>
         </is>
       </c>
       <c r="D27" s="3" t="inlineStr">
         <is>
-          <t>Ra 12,5</t>
-        </is>
-      </c>
-      <c r="E27" s="3" t="n">
-        <v>12.5</v>
-      </c>
+          <t>Грунт ГФ-021, Эмаль ПФ-115 серая</t>
+        </is>
+      </c>
+      <c r="E27" s="3" t="n"/>
       <c r="F27" s="3" t="n"/>
       <c r="G27" s="3" t="n"/>
-      <c r="H27" s="3" t="inlineStr">
-        <is>
-          <t>мкм</t>
-        </is>
-      </c>
+      <c r="H27" s="3" t="n"/>
       <c r="I27" s="3" t="inlineStr">
         <is>
-          <t>Ra</t>
+          <t>Грунт ГФ-021, Эмаль ПФ-115 серая</t>
         </is>
       </c>
       <c r="J27" s="3" t="n"/>
-      <c r="K27" s="3" t="inlineStr">
-        <is>
-          <t>да</t>
-        </is>
-      </c>
+      <c r="K27" s="3" t="inlineStr"/>
       <c r="L27" s="3" t="inlineStr"/>
       <c r="M27" s="3" t="inlineStr">
         <is>
-          <t>√Ra 12,5 (√)</t>
+          <t>Покрытие наружных необработанных поверхностей: Грунт ГФ-021, Эмаль ПФ-115 серая.</t>
         </is>
       </c>
       <c r="N27" s="3" t="inlineStr">
         <is>
-          <t>Чертежи/АРМ.303411.005 Гайка специальная.pdf, стр. 1</t>
+          <t>Чертежи/АРМ.303411.101 Корпус.pdf, стр. 1</t>
         </is>
       </c>
     </row>
@@ -4753,35 +4797,37 @@
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>Общие допуски</t>
+          <t>Допуск размера</t>
         </is>
       </c>
       <c r="D28" s="3" t="inlineStr">
         <is>
-          <t>IT14</t>
-        </is>
-      </c>
-      <c r="E28" s="3" t="n"/>
+          <t>Ø110H7</t>
+        </is>
+      </c>
+      <c r="E28" s="3" t="n">
+        <v>110</v>
+      </c>
       <c r="F28" s="3" t="n"/>
       <c r="G28" s="3" t="n"/>
-      <c r="H28" s="3" t="n"/>
+      <c r="H28" s="3" t="inlineStr">
+        <is>
+          <t>мм</t>
+        </is>
+      </c>
       <c r="I28" s="3" t="inlineStr">
         <is>
-          <t>H14, h14</t>
+          <t>H7</t>
         </is>
       </c>
       <c r="J28" s="3" t="n">
-        <v>14</v>
-      </c>
-      <c r="K28" s="3" t="inlineStr">
-        <is>
-          <t>да</t>
-        </is>
-      </c>
+        <v>7</v>
+      </c>
+      <c r="K28" s="3" t="inlineStr"/>
       <c r="L28" s="3" t="inlineStr"/>
       <c r="M28" s="3" t="inlineStr">
         <is>
-          <t>Неуказанные предельные отклонения размеров: H14, h14, ±IT14/2.</t>
+          <t>Ø110H7</t>
         </is>
       </c>
       <c r="N28" s="3" t="inlineStr">
@@ -4803,29 +4849,37 @@
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>Покрытие</t>
+          <t>Допуск размера</t>
         </is>
       </c>
       <c r="D29" s="3" t="inlineStr">
         <is>
-          <t>Грунт ГФ-021, Эмаль ПФ-115 серая</t>
-        </is>
-      </c>
-      <c r="E29" s="3" t="n"/>
+          <t>Ø90H8</t>
+        </is>
+      </c>
+      <c r="E29" s="3" t="n">
+        <v>90</v>
+      </c>
       <c r="F29" s="3" t="n"/>
       <c r="G29" s="3" t="n"/>
-      <c r="H29" s="3" t="n"/>
+      <c r="H29" s="3" t="inlineStr">
+        <is>
+          <t>мм</t>
+        </is>
+      </c>
       <c r="I29" s="3" t="inlineStr">
         <is>
-          <t>Грунт ГФ-021, Эмаль ПФ-115 серая</t>
-        </is>
-      </c>
-      <c r="J29" s="3" t="n"/>
+          <t>H8</t>
+        </is>
+      </c>
+      <c r="J29" s="3" t="n">
+        <v>8</v>
+      </c>
       <c r="K29" s="3" t="inlineStr"/>
       <c r="L29" s="3" t="inlineStr"/>
       <c r="M29" s="3" t="inlineStr">
         <is>
-          <t>Покрытие наружных необработанных поверхностей: Грунт ГФ-021, Эмаль ПФ-115 серая.</t>
+          <t>Ø90H8</t>
         </is>
       </c>
       <c r="N29" s="3" t="inlineStr">
@@ -4847,37 +4901,35 @@
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>Допуск размера</t>
+          <t>Шероховатость</t>
         </is>
       </c>
       <c r="D30" s="3" t="inlineStr">
         <is>
-          <t>Ø110H7</t>
+          <t>Ra 1,6</t>
         </is>
       </c>
       <c r="E30" s="3" t="n">
-        <v>110</v>
+        <v>1.6</v>
       </c>
       <c r="F30" s="3" t="n"/>
       <c r="G30" s="3" t="n"/>
       <c r="H30" s="3" t="inlineStr">
         <is>
-          <t>мм</t>
+          <t>мкм</t>
         </is>
       </c>
       <c r="I30" s="3" t="inlineStr">
         <is>
-          <t>H7</t>
-        </is>
-      </c>
-      <c r="J30" s="3" t="n">
-        <v>7</v>
-      </c>
+          <t>Ra</t>
+        </is>
+      </c>
+      <c r="J30" s="3" t="n"/>
       <c r="K30" s="3" t="inlineStr"/>
       <c r="L30" s="3" t="inlineStr"/>
       <c r="M30" s="3" t="inlineStr">
         <is>
-          <t>Ø110H7</t>
+          <t>Ra 1,6</t>
         </is>
       </c>
       <c r="N30" s="3" t="inlineStr">
@@ -4899,16 +4951,16 @@
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>Допуск размера</t>
+          <t>Допуск формы/расположения</t>
         </is>
       </c>
       <c r="D31" s="3" t="inlineStr">
         <is>
-          <t>Ø90H8</t>
+          <t>◎ соосности</t>
         </is>
       </c>
       <c r="E31" s="3" t="n">
-        <v>90</v>
+        <v>0.03</v>
       </c>
       <c r="F31" s="3" t="n"/>
       <c r="G31" s="3" t="n"/>
@@ -4919,17 +4971,15 @@
       </c>
       <c r="I31" s="3" t="inlineStr">
         <is>
-          <t>H8</t>
-        </is>
-      </c>
-      <c r="J31" s="3" t="n">
-        <v>8</v>
-      </c>
+          <t>А</t>
+        </is>
+      </c>
+      <c r="J31" s="3" t="n"/>
       <c r="K31" s="3" t="inlineStr"/>
       <c r="L31" s="3" t="inlineStr"/>
       <c r="M31" s="3" t="inlineStr">
         <is>
-          <t>Ø90H8</t>
+          <t>◎ Ø0,03 А</t>
         </is>
       </c>
       <c r="N31" s="3" t="inlineStr">
@@ -4951,27 +5001,27 @@
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>Шероховатость</t>
+          <t>Допуск формы/расположения</t>
         </is>
       </c>
       <c r="D32" s="3" t="inlineStr">
         <is>
-          <t>Ra 1,6</t>
+          <t>∥ параллельности</t>
         </is>
       </c>
       <c r="E32" s="3" t="n">
-        <v>1.6</v>
+        <v>0.05</v>
       </c>
       <c r="F32" s="3" t="n"/>
       <c r="G32" s="3" t="n"/>
       <c r="H32" s="3" t="inlineStr">
         <is>
-          <t>мкм</t>
+          <t>мм</t>
         </is>
       </c>
       <c r="I32" s="3" t="inlineStr">
         <is>
-          <t>Ra</t>
+          <t>Б</t>
         </is>
       </c>
       <c r="J32" s="3" t="n"/>
@@ -4979,7 +5029,7 @@
       <c r="L32" s="3" t="inlineStr"/>
       <c r="M32" s="3" t="inlineStr">
         <is>
-          <t>Ra 1,6</t>
+          <t>∥ 0,05 Б</t>
         </is>
       </c>
       <c r="N32" s="3" t="inlineStr">
@@ -5001,35 +5051,39 @@
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t>Допуск формы/расположения</t>
+          <t>Шероховатость</t>
         </is>
       </c>
       <c r="D33" s="3" t="inlineStr">
         <is>
-          <t>◎ соосности</t>
+          <t>Ra 12,5</t>
         </is>
       </c>
       <c r="E33" s="3" t="n">
-        <v>0.03</v>
+        <v>12.5</v>
       </c>
       <c r="F33" s="3" t="n"/>
       <c r="G33" s="3" t="n"/>
       <c r="H33" s="3" t="inlineStr">
         <is>
-          <t>мм</t>
+          <t>мкм</t>
         </is>
       </c>
       <c r="I33" s="3" t="inlineStr">
         <is>
-          <t>А</t>
+          <t>Ra</t>
         </is>
       </c>
       <c r="J33" s="3" t="n"/>
-      <c r="K33" s="3" t="inlineStr"/>
+      <c r="K33" s="3" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
       <c r="L33" s="3" t="inlineStr"/>
       <c r="M33" s="3" t="inlineStr">
         <is>
-          <t>◎ Ø0,03 А</t>
+          <t>√Ra 12,5 (√)</t>
         </is>
       </c>
       <c r="N33" s="3" t="inlineStr">
@@ -5041,104 +5095,94 @@
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
         <is>
-          <t>АРМ.303411.101</t>
+          <t>АРМ.303411.102</t>
         </is>
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>Корпус</t>
+          <t>Крышка</t>
         </is>
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>Допуск формы/расположения</t>
+          <t>Общие допуски</t>
         </is>
       </c>
       <c r="D34" s="3" t="inlineStr">
         <is>
-          <t>∥ параллельности</t>
-        </is>
-      </c>
-      <c r="E34" s="3" t="n">
-        <v>0.05</v>
-      </c>
+          <t>IT14</t>
+        </is>
+      </c>
+      <c r="E34" s="3" t="n"/>
       <c r="F34" s="3" t="n"/>
       <c r="G34" s="3" t="n"/>
-      <c r="H34" s="3" t="inlineStr">
-        <is>
-          <t>мм</t>
-        </is>
-      </c>
+      <c r="H34" s="3" t="n"/>
       <c r="I34" s="3" t="inlineStr">
         <is>
-          <t>Б</t>
-        </is>
-      </c>
-      <c r="J34" s="3" t="n"/>
-      <c r="K34" s="3" t="inlineStr"/>
+          <t>H14, h14</t>
+        </is>
+      </c>
+      <c r="J34" s="3" t="n">
+        <v>14</v>
+      </c>
+      <c r="K34" s="3" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
       <c r="L34" s="3" t="inlineStr"/>
       <c r="M34" s="3" t="inlineStr">
         <is>
-          <t>∥ 0,05 Б</t>
+          <t>Неуказанные предельные отклонения размеров: H14, h14, ±IT14/2.</t>
         </is>
       </c>
       <c r="N34" s="3" t="inlineStr">
         <is>
-          <t>Чертежи/АРМ.303411.101 Корпус.pdf, стр. 1</t>
+          <t>Чертежи/АРМ.303411.102 Крышка.pdf, стр. 1</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
         <is>
-          <t>АРМ.303411.101</t>
+          <t>АРМ.303411.102</t>
         </is>
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>Корпус</t>
+          <t>Крышка</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>Шероховатость</t>
+          <t>Покрытие</t>
         </is>
       </c>
       <c r="D35" s="3" t="inlineStr">
         <is>
-          <t>Ra 12,5</t>
-        </is>
-      </c>
-      <c r="E35" s="3" t="n">
-        <v>12.5</v>
-      </c>
+          <t>Грунт ГФ-021, Эмаль ПФ-115 серая</t>
+        </is>
+      </c>
+      <c r="E35" s="3" t="n"/>
       <c r="F35" s="3" t="n"/>
       <c r="G35" s="3" t="n"/>
-      <c r="H35" s="3" t="inlineStr">
-        <is>
-          <t>мкм</t>
-        </is>
-      </c>
+      <c r="H35" s="3" t="n"/>
       <c r="I35" s="3" t="inlineStr">
         <is>
-          <t>Ra</t>
+          <t>Грунт ГФ-021, Эмаль ПФ-115 серая</t>
         </is>
       </c>
       <c r="J35" s="3" t="n"/>
-      <c r="K35" s="3" t="inlineStr">
-        <is>
-          <t>да</t>
-        </is>
-      </c>
+      <c r="K35" s="3" t="inlineStr"/>
       <c r="L35" s="3" t="inlineStr"/>
       <c r="M35" s="3" t="inlineStr">
         <is>
-          <t>√Ra 12,5 (√)</t>
+          <t>Покрытие наружных необработанных поверхностей: Грунт ГФ-021, Эмаль ПФ-115 серая.</t>
         </is>
       </c>
       <c r="N35" s="3" t="inlineStr">
         <is>
-          <t>Чертежи/АРМ.303411.101 Корпус.pdf, стр. 1</t>
+          <t>Чертежи/АРМ.303411.102 Крышка.pdf, стр. 1</t>
         </is>
       </c>
     </row>
@@ -5155,35 +5199,37 @@
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>Общие допуски</t>
+          <t>Допуск размера</t>
         </is>
       </c>
       <c r="D36" s="3" t="inlineStr">
         <is>
-          <t>IT14</t>
-        </is>
-      </c>
-      <c r="E36" s="3" t="n"/>
+          <t>Ø110h8</t>
+        </is>
+      </c>
+      <c r="E36" s="3" t="n">
+        <v>110</v>
+      </c>
       <c r="F36" s="3" t="n"/>
       <c r="G36" s="3" t="n"/>
-      <c r="H36" s="3" t="n"/>
+      <c r="H36" s="3" t="inlineStr">
+        <is>
+          <t>мм</t>
+        </is>
+      </c>
       <c r="I36" s="3" t="inlineStr">
         <is>
-          <t>H14, h14</t>
+          <t>h8</t>
         </is>
       </c>
       <c r="J36" s="3" t="n">
-        <v>14</v>
-      </c>
-      <c r="K36" s="3" t="inlineStr">
-        <is>
-          <t>да</t>
-        </is>
-      </c>
+        <v>8</v>
+      </c>
+      <c r="K36" s="3" t="inlineStr"/>
       <c r="L36" s="3" t="inlineStr"/>
       <c r="M36" s="3" t="inlineStr">
         <is>
-          <t>Неуказанные предельные отклонения размеров: H14, h14, ±IT14/2.</t>
+          <t>Ø110h8</t>
         </is>
       </c>
       <c r="N36" s="3" t="inlineStr">
@@ -5205,21 +5251,27 @@
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>Покрытие</t>
+          <t>Шероховатость</t>
         </is>
       </c>
       <c r="D37" s="3" t="inlineStr">
         <is>
-          <t>Грунт ГФ-021, Эмаль ПФ-115 серая</t>
-        </is>
-      </c>
-      <c r="E37" s="3" t="n"/>
+          <t>Ra 3,2</t>
+        </is>
+      </c>
+      <c r="E37" s="3" t="n">
+        <v>3.2</v>
+      </c>
       <c r="F37" s="3" t="n"/>
       <c r="G37" s="3" t="n"/>
-      <c r="H37" s="3" t="n"/>
+      <c r="H37" s="3" t="inlineStr">
+        <is>
+          <t>мкм</t>
+        </is>
+      </c>
       <c r="I37" s="3" t="inlineStr">
         <is>
-          <t>Грунт ГФ-021, Эмаль ПФ-115 серая</t>
+          <t>Ra</t>
         </is>
       </c>
       <c r="J37" s="3" t="n"/>
@@ -5227,7 +5279,7 @@
       <c r="L37" s="3" t="inlineStr"/>
       <c r="M37" s="3" t="inlineStr">
         <is>
-          <t>Покрытие наружных необработанных поверхностей: Грунт ГФ-021, Эмаль ПФ-115 серая.</t>
+          <t>Ra 3,2</t>
         </is>
       </c>
       <c r="N37" s="3" t="inlineStr">
@@ -5249,16 +5301,16 @@
       </c>
       <c r="C38" s="3" t="inlineStr">
         <is>
-          <t>Допуск размера</t>
+          <t>Допуск формы/расположения</t>
         </is>
       </c>
       <c r="D38" s="3" t="inlineStr">
         <is>
-          <t>Ø110h8</t>
+          <t>⏥ плоскостности</t>
         </is>
       </c>
       <c r="E38" s="3" t="n">
-        <v>110</v>
+        <v>0.05</v>
       </c>
       <c r="F38" s="3" t="n"/>
       <c r="G38" s="3" t="n"/>
@@ -5267,19 +5319,13 @@
           <t>мм</t>
         </is>
       </c>
-      <c r="I38" s="3" t="inlineStr">
-        <is>
-          <t>h8</t>
-        </is>
-      </c>
-      <c r="J38" s="3" t="n">
-        <v>8</v>
-      </c>
+      <c r="I38" s="3" t="n"/>
+      <c r="J38" s="3" t="n"/>
       <c r="K38" s="3" t="inlineStr"/>
       <c r="L38" s="3" t="inlineStr"/>
       <c r="M38" s="3" t="inlineStr">
         <is>
-          <t>Ø110h8</t>
+          <t>⏥ 0,05</t>
         </is>
       </c>
       <c r="N38" s="3" t="inlineStr">
@@ -5306,11 +5352,11 @@
       </c>
       <c r="D39" s="3" t="inlineStr">
         <is>
-          <t>Ra 3,2</t>
+          <t>Ra 12,5</t>
         </is>
       </c>
       <c r="E39" s="3" t="n">
-        <v>3.2</v>
+        <v>12.5</v>
       </c>
       <c r="F39" s="3" t="n"/>
       <c r="G39" s="3" t="n"/>
@@ -5325,11 +5371,15 @@
         </is>
       </c>
       <c r="J39" s="3" t="n"/>
-      <c r="K39" s="3" t="inlineStr"/>
+      <c r="K39" s="3" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
       <c r="L39" s="3" t="inlineStr"/>
       <c r="M39" s="3" t="inlineStr">
         <is>
-          <t>Ra 3,2</t>
+          <t>√Ra 12,5 (√)</t>
         </is>
       </c>
       <c r="N39" s="3" t="inlineStr">
@@ -5341,100 +5391,104 @@
     <row r="40">
       <c r="A40" s="3" t="inlineStr">
         <is>
-          <t>АРМ.303411.102</t>
+          <t>АРМ.303411.201</t>
         </is>
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>Крышка</t>
+          <t>Вал ведомый</t>
         </is>
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t>Допуск формы/расположения</t>
+          <t>Твёрдость</t>
         </is>
       </c>
       <c r="D40" s="3" t="inlineStr">
         <is>
-          <t>⏥ плоскостности</t>
-        </is>
-      </c>
-      <c r="E40" s="3" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="F40" s="3" t="n"/>
-      <c r="G40" s="3" t="n"/>
+          <t>Твёрдость HB</t>
+        </is>
+      </c>
+      <c r="E40" s="3" t="n"/>
+      <c r="F40" s="3" t="n">
+        <v>269</v>
+      </c>
+      <c r="G40" s="3" t="n">
+        <v>302</v>
+      </c>
       <c r="H40" s="3" t="inlineStr">
         <is>
-          <t>мм</t>
-        </is>
-      </c>
-      <c r="I40" s="3" t="n"/>
+          <t>HB</t>
+        </is>
+      </c>
+      <c r="I40" s="3" t="inlineStr">
+        <is>
+          <t>HB</t>
+        </is>
+      </c>
       <c r="J40" s="3" t="n"/>
       <c r="K40" s="3" t="inlineStr"/>
       <c r="L40" s="3" t="inlineStr"/>
       <c r="M40" s="3" t="inlineStr">
         <is>
-          <t>⏥ 0,05</t>
+          <t>269...302 HB.</t>
         </is>
       </c>
       <c r="N40" s="3" t="inlineStr">
         <is>
-          <t>Чертежи/АРМ.303411.102 Крышка.pdf, стр. 1</t>
+          <t>Чертежи/АРМ.303411.201 Вал ведомый.pdf, стр. 1</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
         <is>
-          <t>АРМ.303411.102</t>
+          <t>АРМ.303411.201</t>
         </is>
       </c>
       <c r="B41" s="3" t="inlineStr">
         <is>
-          <t>Крышка</t>
+          <t>Вал ведомый</t>
         </is>
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>Шероховатость</t>
+          <t>Термообработка</t>
         </is>
       </c>
       <c r="D41" s="3" t="inlineStr">
         <is>
-          <t>Ra 12,5</t>
-        </is>
-      </c>
-      <c r="E41" s="3" t="n">
-        <v>12.5</v>
-      </c>
-      <c r="F41" s="3" t="n"/>
-      <c r="G41" s="3" t="n"/>
+          <t>Закалка ТВЧ</t>
+        </is>
+      </c>
+      <c r="E41" s="3" t="n"/>
+      <c r="F41" s="3" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="G41" s="3" t="n">
+        <v>2</v>
+      </c>
       <c r="H41" s="3" t="inlineStr">
         <is>
-          <t>мкм</t>
+          <t>мм</t>
         </is>
       </c>
       <c r="I41" s="3" t="inlineStr">
         <is>
-          <t>Ra</t>
+          <t>Закалка ТВЧ</t>
         </is>
       </c>
       <c r="J41" s="3" t="n"/>
-      <c r="K41" s="3" t="inlineStr">
-        <is>
-          <t>да</t>
-        </is>
-      </c>
+      <c r="K41" s="3" t="inlineStr"/>
       <c r="L41" s="3" t="inlineStr"/>
       <c r="M41" s="3" t="inlineStr">
         <is>
-          <t>√Ra 12,5 (√)</t>
+          <t>Поверхности Б закалить ТВЧ h 1,5...2,0 мм, 48...53 HRC.</t>
         </is>
       </c>
       <c r="N41" s="3" t="inlineStr">
         <is>
-          <t>Чертежи/АРМ.303411.102 Крышка.pdf, стр. 1</t>
+          <t>Чертежи/АРМ.303411.201 Вал ведомый.pdf, стр. 1</t>
         </is>
       </c>
     </row>
@@ -5456,32 +5510,36 @@
       </c>
       <c r="D42" s="3" t="inlineStr">
         <is>
-          <t>Твёрдость HB</t>
+          <t>Твёрдость HRC</t>
         </is>
       </c>
       <c r="E42" s="3" t="n"/>
       <c r="F42" s="3" t="n">
-        <v>269</v>
+        <v>48</v>
       </c>
       <c r="G42" s="3" t="n">
-        <v>302</v>
+        <v>53</v>
       </c>
       <c r="H42" s="3" t="inlineStr">
         <is>
-          <t>HB</t>
+          <t>HRC</t>
         </is>
       </c>
       <c r="I42" s="3" t="inlineStr">
         <is>
-          <t>HB</t>
+          <t>HRC</t>
         </is>
       </c>
       <c r="J42" s="3" t="n"/>
       <c r="K42" s="3" t="inlineStr"/>
-      <c r="L42" s="3" t="inlineStr"/>
+      <c r="L42" s="3" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
       <c r="M42" s="3" t="inlineStr">
         <is>
-          <t>269...302 HB.</t>
+          <t>Поверхности Б закалить ТВЧ h 1,5...2,0 мм, 48...53 HRC.</t>
         </is>
       </c>
       <c r="N42" s="3" t="inlineStr">
@@ -5503,37 +5561,35 @@
       </c>
       <c r="C43" s="3" t="inlineStr">
         <is>
-          <t>Термообработка</t>
+          <t>Общие допуски</t>
         </is>
       </c>
       <c r="D43" s="3" t="inlineStr">
         <is>
-          <t>Закалка ТВЧ</t>
+          <t>IT14</t>
         </is>
       </c>
       <c r="E43" s="3" t="n"/>
-      <c r="F43" s="3" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="G43" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="H43" s="3" t="inlineStr">
-        <is>
-          <t>мм</t>
-        </is>
-      </c>
+      <c r="F43" s="3" t="n"/>
+      <c r="G43" s="3" t="n"/>
+      <c r="H43" s="3" t="n"/>
       <c r="I43" s="3" t="inlineStr">
         <is>
-          <t>Закалка ТВЧ</t>
-        </is>
-      </c>
-      <c r="J43" s="3" t="n"/>
-      <c r="K43" s="3" t="inlineStr"/>
+          <t>H14, h14</t>
+        </is>
+      </c>
+      <c r="J43" s="3" t="n">
+        <v>14</v>
+      </c>
+      <c r="K43" s="3" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
       <c r="L43" s="3" t="inlineStr"/>
       <c r="M43" s="3" t="inlineStr">
         <is>
-          <t>Поверхности Б закалить ТВЧ h 1,5...2,0 мм, 48...53 HRC.</t>
+          <t>Неуказанные предельные отклонения размеров: H14, h14, ±IT14/2.</t>
         </is>
       </c>
       <c r="N43" s="3" t="inlineStr">
@@ -5555,32 +5611,32 @@
       </c>
       <c r="C44" s="3" t="inlineStr">
         <is>
-          <t>Твёрдость</t>
+          <t>Допуск размера</t>
         </is>
       </c>
       <c r="D44" s="3" t="inlineStr">
         <is>
-          <t>Твёрдость HRC</t>
-        </is>
-      </c>
-      <c r="E44" s="3" t="n"/>
-      <c r="F44" s="3" t="n">
-        <v>48</v>
-      </c>
-      <c r="G44" s="3" t="n">
-        <v>53</v>
-      </c>
+          <t>Ø50k6</t>
+        </is>
+      </c>
+      <c r="E44" s="3" t="n">
+        <v>50</v>
+      </c>
+      <c r="F44" s="3" t="n"/>
+      <c r="G44" s="3" t="n"/>
       <c r="H44" s="3" t="inlineStr">
         <is>
-          <t>HRC</t>
+          <t>мм</t>
         </is>
       </c>
       <c r="I44" s="3" t="inlineStr">
         <is>
-          <t>HRC</t>
-        </is>
-      </c>
-      <c r="J44" s="3" t="n"/>
+          <t>k6</t>
+        </is>
+      </c>
+      <c r="J44" s="3" t="n">
+        <v>6</v>
+      </c>
       <c r="K44" s="3" t="inlineStr"/>
       <c r="L44" s="3" t="inlineStr">
         <is>
@@ -5589,7 +5645,7 @@
       </c>
       <c r="M44" s="3" t="inlineStr">
         <is>
-          <t>Поверхности Б закалить ТВЧ h 1,5...2,0 мм, 48...53 HRC.</t>
+          <t>Ø50k6</t>
         </is>
       </c>
       <c r="N44" s="3" t="inlineStr">
@@ -5611,35 +5667,41 @@
       </c>
       <c r="C45" s="3" t="inlineStr">
         <is>
-          <t>Общие допуски</t>
+          <t>Допуск размера</t>
         </is>
       </c>
       <c r="D45" s="3" t="inlineStr">
         <is>
-          <t>IT14</t>
-        </is>
-      </c>
-      <c r="E45" s="3" t="n"/>
+          <t>Ø45h6</t>
+        </is>
+      </c>
+      <c r="E45" s="3" t="n">
+        <v>45</v>
+      </c>
       <c r="F45" s="3" t="n"/>
       <c r="G45" s="3" t="n"/>
-      <c r="H45" s="3" t="n"/>
+      <c r="H45" s="3" t="inlineStr">
+        <is>
+          <t>мм</t>
+        </is>
+      </c>
       <c r="I45" s="3" t="inlineStr">
         <is>
-          <t>H14, h14</t>
+          <t>h6</t>
         </is>
       </c>
       <c r="J45" s="3" t="n">
-        <v>14</v>
-      </c>
-      <c r="K45" s="3" t="inlineStr">
+        <v>6</v>
+      </c>
+      <c r="K45" s="3" t="inlineStr"/>
+      <c r="L45" s="3" t="inlineStr">
         <is>
           <t>да</t>
         </is>
       </c>
-      <c r="L45" s="3" t="inlineStr"/>
       <c r="M45" s="3" t="inlineStr">
         <is>
-          <t>Неуказанные предельные отклонения размеров: H14, h14, ±IT14/2.</t>
+          <t>Ø45h6</t>
         </is>
       </c>
       <c r="N45" s="3" t="inlineStr">
@@ -5666,11 +5728,11 @@
       </c>
       <c r="D46" s="3" t="inlineStr">
         <is>
-          <t>Ø50k6</t>
+          <t>16N9</t>
         </is>
       </c>
       <c r="E46" s="3" t="n">
-        <v>50</v>
+        <v>16</v>
       </c>
       <c r="F46" s="3" t="n"/>
       <c r="G46" s="3" t="n"/>
@@ -5681,21 +5743,17 @@
       </c>
       <c r="I46" s="3" t="inlineStr">
         <is>
-          <t>k6</t>
+          <t>N9</t>
         </is>
       </c>
       <c r="J46" s="3" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="K46" s="3" t="inlineStr"/>
-      <c r="L46" s="3" t="inlineStr">
-        <is>
-          <t>да</t>
-        </is>
-      </c>
+      <c r="L46" s="3" t="inlineStr"/>
       <c r="M46" s="3" t="inlineStr">
         <is>
-          <t>Ø50k6</t>
+          <t>16N9</t>
         </is>
       </c>
       <c r="N46" s="3" t="inlineStr">
@@ -5717,32 +5775,30 @@
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t>Допуск размера</t>
+          <t>Шероховатость</t>
         </is>
       </c>
       <c r="D47" s="3" t="inlineStr">
         <is>
-          <t>Ø45h6</t>
+          <t>Ra 0,8</t>
         </is>
       </c>
       <c r="E47" s="3" t="n">
-        <v>45</v>
+        <v>0.8</v>
       </c>
       <c r="F47" s="3" t="n"/>
       <c r="G47" s="3" t="n"/>
       <c r="H47" s="3" t="inlineStr">
         <is>
-          <t>мм</t>
+          <t>мкм</t>
         </is>
       </c>
       <c r="I47" s="3" t="inlineStr">
         <is>
-          <t>h6</t>
-        </is>
-      </c>
-      <c r="J47" s="3" t="n">
-        <v>6</v>
-      </c>
+          <t>Ra</t>
+        </is>
+      </c>
+      <c r="J47" s="3" t="n"/>
       <c r="K47" s="3" t="inlineStr"/>
       <c r="L47" s="3" t="inlineStr">
         <is>
@@ -5751,7 +5807,7 @@
       </c>
       <c r="M47" s="3" t="inlineStr">
         <is>
-          <t>Ø45h6</t>
+          <t>Ra 0,8</t>
         </is>
       </c>
       <c r="N47" s="3" t="inlineStr">
@@ -5773,37 +5829,35 @@
       </c>
       <c r="C48" s="3" t="inlineStr">
         <is>
-          <t>Допуск размера</t>
+          <t>Шероховатость</t>
         </is>
       </c>
       <c r="D48" s="3" t="inlineStr">
         <is>
-          <t>16N9</t>
+          <t>Ra 1,6</t>
         </is>
       </c>
       <c r="E48" s="3" t="n">
-        <v>16</v>
+        <v>1.6</v>
       </c>
       <c r="F48" s="3" t="n"/>
       <c r="G48" s="3" t="n"/>
       <c r="H48" s="3" t="inlineStr">
         <is>
-          <t>мм</t>
+          <t>мкм</t>
         </is>
       </c>
       <c r="I48" s="3" t="inlineStr">
         <is>
-          <t>N9</t>
-        </is>
-      </c>
-      <c r="J48" s="3" t="n">
-        <v>9</v>
-      </c>
+          <t>Ra</t>
+        </is>
+      </c>
+      <c r="J48" s="3" t="n"/>
       <c r="K48" s="3" t="inlineStr"/>
       <c r="L48" s="3" t="inlineStr"/>
       <c r="M48" s="3" t="inlineStr">
         <is>
-          <t>16N9</t>
+          <t>Ra 1,6</t>
         </is>
       </c>
       <c r="N48" s="3" t="inlineStr">
@@ -5825,27 +5879,27 @@
       </c>
       <c r="C49" s="3" t="inlineStr">
         <is>
-          <t>Шероховатость</t>
+          <t>Допуск формы/расположения</t>
         </is>
       </c>
       <c r="D49" s="3" t="inlineStr">
         <is>
-          <t>Ra 0,8</t>
+          <t>↗ биения</t>
         </is>
       </c>
       <c r="E49" s="3" t="n">
-        <v>0.8</v>
+        <v>0.016</v>
       </c>
       <c r="F49" s="3" t="n"/>
       <c r="G49" s="3" t="n"/>
       <c r="H49" s="3" t="inlineStr">
         <is>
-          <t>мкм</t>
+          <t>мм</t>
         </is>
       </c>
       <c r="I49" s="3" t="inlineStr">
         <is>
-          <t>Ra</t>
+          <t>А-Б</t>
         </is>
       </c>
       <c r="J49" s="3" t="n"/>
@@ -5857,7 +5911,7 @@
       </c>
       <c r="M49" s="3" t="inlineStr">
         <is>
-          <t>Ra 0,8</t>
+          <t>↗ 0,016 А-Б</t>
         </is>
       </c>
       <c r="N49" s="3" t="inlineStr">
@@ -5884,11 +5938,11 @@
       </c>
       <c r="D50" s="3" t="inlineStr">
         <is>
-          <t>Ra 1,6</t>
+          <t>Ra 6,3</t>
         </is>
       </c>
       <c r="E50" s="3" t="n">
-        <v>1.6</v>
+        <v>6.3</v>
       </c>
       <c r="F50" s="3" t="n"/>
       <c r="G50" s="3" t="n"/>
@@ -5903,11 +5957,15 @@
         </is>
       </c>
       <c r="J50" s="3" t="n"/>
-      <c r="K50" s="3" t="inlineStr"/>
+      <c r="K50" s="3" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
       <c r="L50" s="3" t="inlineStr"/>
       <c r="M50" s="3" t="inlineStr">
         <is>
-          <t>Ra 1,6</t>
+          <t>√Ra 6,3 (√)</t>
         </is>
       </c>
       <c r="N50" s="3" t="inlineStr">
@@ -5919,29 +5977,31 @@
     <row r="51">
       <c r="A51" s="3" t="inlineStr">
         <is>
-          <t>АРМ.303411.201</t>
+          <t>АРМ.303411.202</t>
         </is>
       </c>
       <c r="B51" s="3" t="inlineStr">
         <is>
-          <t>Вал ведомый</t>
+          <t>Колесо зубчатое</t>
         </is>
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>Допуск формы/расположения</t>
+          <t>Термообработка</t>
         </is>
       </c>
       <c r="D51" s="3" t="inlineStr">
         <is>
-          <t>↗ биения</t>
-        </is>
-      </c>
-      <c r="E51" s="3" t="n">
-        <v>0.016</v>
-      </c>
-      <c r="F51" s="3" t="n"/>
-      <c r="G51" s="3" t="n"/>
+          <t>Цементация</t>
+        </is>
+      </c>
+      <c r="E51" s="3" t="n"/>
+      <c r="F51" s="3" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="G51" s="3" t="n">
+        <v>1.2</v>
+      </c>
       <c r="H51" s="3" t="inlineStr">
         <is>
           <t>мм</t>
@@ -5949,7 +6009,7 @@
       </c>
       <c r="I51" s="3" t="inlineStr">
         <is>
-          <t>А-Б</t>
+          <t>Цементация</t>
         </is>
       </c>
       <c r="J51" s="3" t="n"/>
@@ -5961,66 +6021,68 @@
       </c>
       <c r="M51" s="3" t="inlineStr">
         <is>
-          <t>↗ 0,016 А-Б</t>
+          <t>Цементировать h 0,8...1,2 мм, 58...62 HRC.</t>
         </is>
       </c>
       <c r="N51" s="3" t="inlineStr">
         <is>
-          <t>Чертежи/АРМ.303411.201 Вал ведомый.pdf, стр. 1</t>
+          <t>Чертежи/АРМ.303411.202 Колесо зубчатое.pdf, стр. 1</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="3" t="inlineStr">
         <is>
-          <t>АРМ.303411.201</t>
+          <t>АРМ.303411.202</t>
         </is>
       </c>
       <c r="B52" s="3" t="inlineStr">
         <is>
-          <t>Вал ведомый</t>
+          <t>Колесо зубчатое</t>
         </is>
       </c>
       <c r="C52" s="3" t="inlineStr">
         <is>
-          <t>Шероховатость</t>
+          <t>Твёрдость</t>
         </is>
       </c>
       <c r="D52" s="3" t="inlineStr">
         <is>
-          <t>Ra 6,3</t>
-        </is>
-      </c>
-      <c r="E52" s="3" t="n">
-        <v>6.3</v>
-      </c>
-      <c r="F52" s="3" t="n"/>
-      <c r="G52" s="3" t="n"/>
+          <t>Твёрдость HRC</t>
+        </is>
+      </c>
+      <c r="E52" s="3" t="n"/>
+      <c r="F52" s="3" t="n">
+        <v>58</v>
+      </c>
+      <c r="G52" s="3" t="n">
+        <v>62</v>
+      </c>
       <c r="H52" s="3" t="inlineStr">
         <is>
-          <t>мкм</t>
+          <t>HRC</t>
         </is>
       </c>
       <c r="I52" s="3" t="inlineStr">
         <is>
-          <t>Ra</t>
+          <t>HRC</t>
         </is>
       </c>
       <c r="J52" s="3" t="n"/>
-      <c r="K52" s="3" t="inlineStr">
+      <c r="K52" s="3" t="inlineStr"/>
+      <c r="L52" s="3" t="inlineStr">
         <is>
           <t>да</t>
         </is>
       </c>
-      <c r="L52" s="3" t="inlineStr"/>
       <c r="M52" s="3" t="inlineStr">
         <is>
-          <t>√Ra 6,3 (√)</t>
+          <t>Цементировать h 0,8...1,2 мм, 58...62 HRC.</t>
         </is>
       </c>
       <c r="N52" s="3" t="inlineStr">
         <is>
-          <t>Чертежи/АРМ.303411.201 Вал ведомый.pdf, стр. 1</t>
+          <t>Чертежи/АРМ.303411.202 Колесо зубчатое.pdf, стр. 1</t>
         </is>
       </c>
     </row>
@@ -6037,41 +6099,35 @@
       </c>
       <c r="C53" s="3" t="inlineStr">
         <is>
-          <t>Термообработка</t>
+          <t>Общие допуски</t>
         </is>
       </c>
       <c r="D53" s="3" t="inlineStr">
         <is>
-          <t>Цементация</t>
+          <t>IT14</t>
         </is>
       </c>
       <c r="E53" s="3" t="n"/>
-      <c r="F53" s="3" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="G53" s="3" t="n">
-        <v>1.2</v>
-      </c>
-      <c r="H53" s="3" t="inlineStr">
-        <is>
-          <t>мм</t>
-        </is>
-      </c>
+      <c r="F53" s="3" t="n"/>
+      <c r="G53" s="3" t="n"/>
+      <c r="H53" s="3" t="n"/>
       <c r="I53" s="3" t="inlineStr">
         <is>
-          <t>Цементация</t>
-        </is>
-      </c>
-      <c r="J53" s="3" t="n"/>
-      <c r="K53" s="3" t="inlineStr"/>
-      <c r="L53" s="3" t="inlineStr">
+          <t>H14, h14</t>
+        </is>
+      </c>
+      <c r="J53" s="3" t="n">
+        <v>14</v>
+      </c>
+      <c r="K53" s="3" t="inlineStr">
         <is>
           <t>да</t>
         </is>
       </c>
+      <c r="L53" s="3" t="inlineStr"/>
       <c r="M53" s="3" t="inlineStr">
         <is>
-          <t>Цементировать h 0,8...1,2 мм, 58...62 HRC.</t>
+          <t>Неуказанные предельные отклонения размеров: H14, h14, ±IT14/2.</t>
         </is>
       </c>
       <c r="N53" s="3" t="inlineStr">
@@ -6093,41 +6149,37 @@
       </c>
       <c r="C54" s="3" t="inlineStr">
         <is>
-          <t>Твёрдость</t>
+          <t>Допуск размера</t>
         </is>
       </c>
       <c r="D54" s="3" t="inlineStr">
         <is>
-          <t>Твёрдость HRC</t>
-        </is>
-      </c>
-      <c r="E54" s="3" t="n"/>
-      <c r="F54" s="3" t="n">
-        <v>58</v>
-      </c>
-      <c r="G54" s="3" t="n">
-        <v>62</v>
-      </c>
+          <t>Ø50H7</t>
+        </is>
+      </c>
+      <c r="E54" s="3" t="n">
+        <v>50</v>
+      </c>
+      <c r="F54" s="3" t="n"/>
+      <c r="G54" s="3" t="n"/>
       <c r="H54" s="3" t="inlineStr">
         <is>
-          <t>HRC</t>
+          <t>мм</t>
         </is>
       </c>
       <c r="I54" s="3" t="inlineStr">
         <is>
-          <t>HRC</t>
-        </is>
-      </c>
-      <c r="J54" s="3" t="n"/>
+          <t>H7</t>
+        </is>
+      </c>
+      <c r="J54" s="3" t="n">
+        <v>7</v>
+      </c>
       <c r="K54" s="3" t="inlineStr"/>
-      <c r="L54" s="3" t="inlineStr">
-        <is>
-          <t>да</t>
-        </is>
-      </c>
+      <c r="L54" s="3" t="inlineStr"/>
       <c r="M54" s="3" t="inlineStr">
         <is>
-          <t>Цементировать h 0,8...1,2 мм, 58...62 HRC.</t>
+          <t>Ø50H7</t>
         </is>
       </c>
       <c r="N54" s="3" t="inlineStr">
@@ -6149,35 +6201,37 @@
       </c>
       <c r="C55" s="3" t="inlineStr">
         <is>
-          <t>Общие допуски</t>
+          <t>Допуск размера</t>
         </is>
       </c>
       <c r="D55" s="3" t="inlineStr">
         <is>
-          <t>IT14</t>
-        </is>
-      </c>
-      <c r="E55" s="3" t="n"/>
+          <t>16Js9</t>
+        </is>
+      </c>
+      <c r="E55" s="3" t="n">
+        <v>16</v>
+      </c>
       <c r="F55" s="3" t="n"/>
       <c r="G55" s="3" t="n"/>
-      <c r="H55" s="3" t="n"/>
+      <c r="H55" s="3" t="inlineStr">
+        <is>
+          <t>мм</t>
+        </is>
+      </c>
       <c r="I55" s="3" t="inlineStr">
         <is>
-          <t>H14, h14</t>
+          <t>Js9</t>
         </is>
       </c>
       <c r="J55" s="3" t="n">
-        <v>14</v>
-      </c>
-      <c r="K55" s="3" t="inlineStr">
-        <is>
-          <t>да</t>
-        </is>
-      </c>
+        <v>9</v>
+      </c>
+      <c r="K55" s="3" t="inlineStr"/>
       <c r="L55" s="3" t="inlineStr"/>
       <c r="M55" s="3" t="inlineStr">
         <is>
-          <t>Неуказанные предельные отклонения размеров: H14, h14, ±IT14/2.</t>
+          <t>16Js9</t>
         </is>
       </c>
       <c r="N55" s="3" t="inlineStr">
@@ -6199,37 +6253,39 @@
       </c>
       <c r="C56" s="3" t="inlineStr">
         <is>
-          <t>Допуск размера</t>
+          <t>Шероховатость</t>
         </is>
       </c>
       <c r="D56" s="3" t="inlineStr">
         <is>
-          <t>Ø50H7</t>
+          <t>Ra 0,4</t>
         </is>
       </c>
       <c r="E56" s="3" t="n">
-        <v>50</v>
+        <v>0.4</v>
       </c>
       <c r="F56" s="3" t="n"/>
       <c r="G56" s="3" t="n"/>
       <c r="H56" s="3" t="inlineStr">
         <is>
-          <t>мм</t>
+          <t>мкм</t>
         </is>
       </c>
       <c r="I56" s="3" t="inlineStr">
         <is>
-          <t>H7</t>
-        </is>
-      </c>
-      <c r="J56" s="3" t="n">
-        <v>7</v>
-      </c>
+          <t>Ra</t>
+        </is>
+      </c>
+      <c r="J56" s="3" t="n"/>
       <c r="K56" s="3" t="inlineStr"/>
-      <c r="L56" s="3" t="inlineStr"/>
+      <c r="L56" s="3" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
       <c r="M56" s="3" t="inlineStr">
         <is>
-          <t>Ø50H7</t>
+          <t>Ra 0,4</t>
         </is>
       </c>
       <c r="N56" s="3" t="inlineStr">
@@ -6251,37 +6307,39 @@
       </c>
       <c r="C57" s="3" t="inlineStr">
         <is>
-          <t>Допуск размера</t>
+          <t>Шероховатость</t>
         </is>
       </c>
       <c r="D57" s="3" t="inlineStr">
         <is>
-          <t>16Js9</t>
+          <t>Ra 0,8</t>
         </is>
       </c>
       <c r="E57" s="3" t="n">
-        <v>16</v>
+        <v>0.8</v>
       </c>
       <c r="F57" s="3" t="n"/>
       <c r="G57" s="3" t="n"/>
       <c r="H57" s="3" t="inlineStr">
         <is>
-          <t>мм</t>
+          <t>мкм</t>
         </is>
       </c>
       <c r="I57" s="3" t="inlineStr">
         <is>
-          <t>Js9</t>
-        </is>
-      </c>
-      <c r="J57" s="3" t="n">
-        <v>9</v>
-      </c>
+          <t>Ra</t>
+        </is>
+      </c>
+      <c r="J57" s="3" t="n"/>
       <c r="K57" s="3" t="inlineStr"/>
-      <c r="L57" s="3" t="inlineStr"/>
+      <c r="L57" s="3" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
       <c r="M57" s="3" t="inlineStr">
         <is>
-          <t>16Js9</t>
+          <t>Ra 0,8</t>
         </is>
       </c>
       <c r="N57" s="3" t="inlineStr">
@@ -6303,27 +6361,27 @@
       </c>
       <c r="C58" s="3" t="inlineStr">
         <is>
-          <t>Шероховатость</t>
+          <t>Допуск формы/расположения</t>
         </is>
       </c>
       <c r="D58" s="3" t="inlineStr">
         <is>
-          <t>Ra 0,4</t>
+          <t>↗ биения</t>
         </is>
       </c>
       <c r="E58" s="3" t="n">
-        <v>0.4</v>
+        <v>0.02</v>
       </c>
       <c r="F58" s="3" t="n"/>
       <c r="G58" s="3" t="n"/>
       <c r="H58" s="3" t="inlineStr">
         <is>
-          <t>мкм</t>
+          <t>мм</t>
         </is>
       </c>
       <c r="I58" s="3" t="inlineStr">
         <is>
-          <t>Ra</t>
+          <t>А</t>
         </is>
       </c>
       <c r="J58" s="3" t="n"/>
@@ -6335,7 +6393,7 @@
       </c>
       <c r="M58" s="3" t="inlineStr">
         <is>
-          <t>Ra 0,4</t>
+          <t>↗ 0,02 А</t>
         </is>
       </c>
       <c r="N58" s="3" t="inlineStr">
@@ -6362,11 +6420,11 @@
       </c>
       <c r="D59" s="3" t="inlineStr">
         <is>
-          <t>Ra 0,8</t>
+          <t>Ra 6,3</t>
         </is>
       </c>
       <c r="E59" s="3" t="n">
-        <v>0.8</v>
+        <v>6.3</v>
       </c>
       <c r="F59" s="3" t="n"/>
       <c r="G59" s="3" t="n"/>
@@ -6381,15 +6439,15 @@
         </is>
       </c>
       <c r="J59" s="3" t="n"/>
-      <c r="K59" s="3" t="inlineStr"/>
-      <c r="L59" s="3" t="inlineStr">
+      <c r="K59" s="3" t="inlineStr">
         <is>
           <t>да</t>
         </is>
       </c>
+      <c r="L59" s="3" t="inlineStr"/>
       <c r="M59" s="3" t="inlineStr">
         <is>
-          <t>Ra 0,8</t>
+          <t>√Ra 6,3 (√)</t>
         </is>
       </c>
       <c r="N59" s="3" t="inlineStr">
@@ -6401,26 +6459,26 @@
     <row r="60">
       <c r="A60" s="3" t="inlineStr">
         <is>
-          <t>АРМ.303411.202</t>
+          <t>АРМ.303411.203</t>
         </is>
       </c>
       <c r="B60" s="3" t="inlineStr">
         <is>
-          <t>Колесо зубчатое</t>
+          <t>Кольцо распорное</t>
         </is>
       </c>
       <c r="C60" s="3" t="inlineStr">
         <is>
-          <t>Допуск формы/расположения</t>
+          <t>Допуск размера</t>
         </is>
       </c>
       <c r="D60" s="3" t="inlineStr">
         <is>
-          <t>↗ биения</t>
+          <t>0H9</t>
         </is>
       </c>
       <c r="E60" s="3" t="n">
-        <v>0.02</v>
+        <v>0</v>
       </c>
       <c r="F60" s="3" t="n"/>
       <c r="G60" s="3" t="n"/>
@@ -6431,36 +6489,34 @@
       </c>
       <c r="I60" s="3" t="inlineStr">
         <is>
-          <t>А</t>
-        </is>
-      </c>
-      <c r="J60" s="3" t="n"/>
+          <t>H9</t>
+        </is>
+      </c>
+      <c r="J60" s="3" t="n">
+        <v>9</v>
+      </c>
       <c r="K60" s="3" t="inlineStr"/>
-      <c r="L60" s="3" t="inlineStr">
-        <is>
-          <t>да</t>
-        </is>
-      </c>
+      <c r="L60" s="3" t="inlineStr"/>
       <c r="M60" s="3" t="inlineStr">
         <is>
-          <t>↗ 0,02 А</t>
+          <t>@S0H9</t>
         </is>
       </c>
       <c r="N60" s="3" t="inlineStr">
         <is>
-          <t>Чертежи/АРМ.303411.202 Колесо зубчатое.pdf, стр. 1</t>
+          <t>Чертежи/АРМ.303411.203.jpg, стр. 1</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="3" t="inlineStr">
         <is>
-          <t>АРМ.303411.202</t>
+          <t>АРМ.303411.203</t>
         </is>
       </c>
       <c r="B61" s="3" t="inlineStr">
         <is>
-          <t>Колесо зубчатое</t>
+          <t>Кольцо распорное</t>
         </is>
       </c>
       <c r="C61" s="3" t="inlineStr">
@@ -6470,11 +6526,11 @@
       </c>
       <c r="D61" s="3" t="inlineStr">
         <is>
-          <t>Ra 6,3</t>
+          <t>Ra 3,2</t>
         </is>
       </c>
       <c r="E61" s="3" t="n">
-        <v>6.3</v>
+        <v>3.2</v>
       </c>
       <c r="F61" s="3" t="n"/>
       <c r="G61" s="3" t="n"/>
@@ -6489,122 +6545,110 @@
         </is>
       </c>
       <c r="J61" s="3" t="n"/>
-      <c r="K61" s="3" t="inlineStr">
-        <is>
-          <t>да</t>
-        </is>
-      </c>
+      <c r="K61" s="3" t="inlineStr"/>
       <c r="L61" s="3" t="inlineStr"/>
       <c r="M61" s="3" t="inlineStr">
         <is>
-          <t>√Ra 6,3 (√)</t>
+          <t>Ra 3,2</t>
         </is>
       </c>
       <c r="N61" s="3" t="inlineStr">
         <is>
-          <t>Чертежи/АРМ.303411.202 Колесо зубчатое.pdf, стр. 1</t>
+          <t>Чертежи/АРМ.303411.203.jpg, стр. 1</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="3" t="inlineStr">
         <is>
-          <t>АРМ.303411.203</t>
+          <t>АРМ.303412.007</t>
         </is>
       </c>
       <c r="B62" s="3" t="inlineStr">
         <is>
-          <t>Кольцо распорное</t>
+          <t>Кронштейн</t>
         </is>
       </c>
       <c r="C62" s="3" t="inlineStr">
         <is>
-          <t>Допуск размера</t>
+          <t>Покрытие</t>
         </is>
       </c>
       <c r="D62" s="3" t="inlineStr">
         <is>
-          <t>50H9</t>
-        </is>
-      </c>
-      <c r="E62" s="3" t="n">
-        <v>50</v>
-      </c>
+          <t>Грунт ГФ-021, Эмаль ПФ-115 серая</t>
+        </is>
+      </c>
+      <c r="E62" s="3" t="n"/>
       <c r="F62" s="3" t="n"/>
       <c r="G62" s="3" t="n"/>
-      <c r="H62" s="3" t="inlineStr">
-        <is>
-          <t>мм</t>
-        </is>
-      </c>
+      <c r="H62" s="3" t="n"/>
       <c r="I62" s="3" t="inlineStr">
         <is>
-          <t>H9</t>
-        </is>
-      </c>
-      <c r="J62" s="3" t="n">
-        <v>9</v>
-      </c>
+          <t>Грунт ГФ-021, Эмаль ПФ-115 серая</t>
+        </is>
+      </c>
+      <c r="J62" s="3" t="n"/>
       <c r="K62" s="3" t="inlineStr"/>
       <c r="L62" s="3" t="inlineStr"/>
       <c r="M62" s="3" t="inlineStr">
         <is>
-          <t>@50H9</t>
+          <t>Покрытие: Грунт ГФ-021, Эмаль ПФ-115 серая.</t>
         </is>
       </c>
       <c r="N62" s="3" t="inlineStr">
         <is>
-          <t>Чертежи/АРМ.303411.203.jpg, стр. 1</t>
+          <t>Чертежи/АРМ.303412.007 Кронштейн.pdf, стр. 1</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="3" t="inlineStr">
         <is>
-          <t>АРМ.303411.203</t>
+          <t>АРМ.303412.007</t>
         </is>
       </c>
       <c r="B63" s="3" t="inlineStr">
         <is>
-          <t>Кольцо распорное</t>
+          <t>Кронштейн</t>
         </is>
       </c>
       <c r="C63" s="3" t="inlineStr">
         <is>
-          <t>Шероховатость</t>
+          <t>Общие допуски</t>
         </is>
       </c>
       <c r="D63" s="3" t="inlineStr">
         <is>
-          <t>Ra 3,2</t>
-        </is>
-      </c>
-      <c r="E63" s="3" t="n">
-        <v>3.2</v>
-      </c>
+          <t>IT14</t>
+        </is>
+      </c>
+      <c r="E63" s="3" t="n"/>
       <c r="F63" s="3" t="n"/>
       <c r="G63" s="3" t="n"/>
-      <c r="H63" s="3" t="inlineStr">
-        <is>
-          <t>мкм</t>
-        </is>
-      </c>
+      <c r="H63" s="3" t="n"/>
       <c r="I63" s="3" t="inlineStr">
         <is>
-          <t>Ra</t>
-        </is>
-      </c>
-      <c r="J63" s="3" t="n"/>
-      <c r="K63" s="3" t="inlineStr"/>
+          <t>H14, h14</t>
+        </is>
+      </c>
+      <c r="J63" s="3" t="n">
+        <v>14</v>
+      </c>
+      <c r="K63" s="3" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
       <c r="L63" s="3" t="inlineStr"/>
       <c r="M63" s="3" t="inlineStr">
         <is>
-          <t>Ва 3,2</t>
+          <t>Неуказанные предельные отклонения размеров: H14, h14, ±IT14/2.</t>
         </is>
       </c>
       <c r="N63" s="3" t="inlineStr">
         <is>
-          <t>Чертежи/АРМ.303411.203.jpg, стр. 1</t>
+          <t>Чертежи/АРМ.303412.007 Кронштейн.pdf, стр. 1</t>
         </is>
       </c>
     </row>
@@ -6621,29 +6665,37 @@
       </c>
       <c r="C64" s="3" t="inlineStr">
         <is>
-          <t>Покрытие</t>
+          <t>Допуск размера</t>
         </is>
       </c>
       <c r="D64" s="3" t="inlineStr">
         <is>
-          <t>Грунт ГФ-021, Эмаль ПФ-115 серая</t>
-        </is>
-      </c>
-      <c r="E64" s="3" t="n"/>
+          <t>Ø18H12</t>
+        </is>
+      </c>
+      <c r="E64" s="3" t="n">
+        <v>18</v>
+      </c>
       <c r="F64" s="3" t="n"/>
       <c r="G64" s="3" t="n"/>
-      <c r="H64" s="3" t="n"/>
+      <c r="H64" s="3" t="inlineStr">
+        <is>
+          <t>мм</t>
+        </is>
+      </c>
       <c r="I64" s="3" t="inlineStr">
         <is>
-          <t>Грунт ГФ-021, Эмаль ПФ-115 серая</t>
-        </is>
-      </c>
-      <c r="J64" s="3" t="n"/>
+          <t>H12</t>
+        </is>
+      </c>
+      <c r="J64" s="3" t="n">
+        <v>12</v>
+      </c>
       <c r="K64" s="3" t="inlineStr"/>
       <c r="L64" s="3" t="inlineStr"/>
       <c r="M64" s="3" t="inlineStr">
         <is>
-          <t>Покрытие: Грунт ГФ-021, Эмаль ПФ-115 серая.</t>
+          <t>Ø18H12</t>
         </is>
       </c>
       <c r="N64" s="3" t="inlineStr">
@@ -6665,35 +6717,35 @@
       </c>
       <c r="C65" s="3" t="inlineStr">
         <is>
-          <t>Общие допуски</t>
+          <t>Шероховатость</t>
         </is>
       </c>
       <c r="D65" s="3" t="inlineStr">
         <is>
-          <t>IT14</t>
-        </is>
-      </c>
-      <c r="E65" s="3" t="n"/>
+          <t>Ra 12,5</t>
+        </is>
+      </c>
+      <c r="E65" s="3" t="n">
+        <v>12.5</v>
+      </c>
       <c r="F65" s="3" t="n"/>
       <c r="G65" s="3" t="n"/>
-      <c r="H65" s="3" t="n"/>
+      <c r="H65" s="3" t="inlineStr">
+        <is>
+          <t>мкм</t>
+        </is>
+      </c>
       <c r="I65" s="3" t="inlineStr">
         <is>
-          <t>H14, h14</t>
-        </is>
-      </c>
-      <c r="J65" s="3" t="n">
-        <v>14</v>
-      </c>
-      <c r="K65" s="3" t="inlineStr">
-        <is>
-          <t>да</t>
-        </is>
-      </c>
+          <t>Ra</t>
+        </is>
+      </c>
+      <c r="J65" s="3" t="n"/>
+      <c r="K65" s="3" t="inlineStr"/>
       <c r="L65" s="3" t="inlineStr"/>
       <c r="M65" s="3" t="inlineStr">
         <is>
-          <t>Неуказанные предельные отклонения размеров: H14, h14, ±IT14/2.</t>
+          <t>Ra 12,5</t>
         </is>
       </c>
       <c r="N65" s="3" t="inlineStr">
@@ -6715,37 +6767,39 @@
       </c>
       <c r="C66" s="3" t="inlineStr">
         <is>
-          <t>Допуск размера</t>
+          <t>Шероховатость</t>
         </is>
       </c>
       <c r="D66" s="3" t="inlineStr">
         <is>
-          <t>Ø18H12</t>
+          <t>Ra 25</t>
         </is>
       </c>
       <c r="E66" s="3" t="n">
-        <v>18</v>
+        <v>25</v>
       </c>
       <c r="F66" s="3" t="n"/>
       <c r="G66" s="3" t="n"/>
       <c r="H66" s="3" t="inlineStr">
         <is>
-          <t>мм</t>
+          <t>мкм</t>
         </is>
       </c>
       <c r="I66" s="3" t="inlineStr">
         <is>
-          <t>H12</t>
-        </is>
-      </c>
-      <c r="J66" s="3" t="n">
-        <v>12</v>
-      </c>
-      <c r="K66" s="3" t="inlineStr"/>
+          <t>Ra</t>
+        </is>
+      </c>
+      <c r="J66" s="3" t="n"/>
+      <c r="K66" s="3" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
       <c r="L66" s="3" t="inlineStr"/>
       <c r="M66" s="3" t="inlineStr">
         <is>
-          <t>Ø18H12</t>
+          <t>√Ra 25 (√)</t>
         </is>
       </c>
       <c r="N66" s="3" t="inlineStr">
@@ -6757,37 +6811,39 @@
     <row r="67">
       <c r="A67" s="3" t="inlineStr">
         <is>
-          <t>АРМ.303412.007</t>
+          <t>АРМ.303411.201</t>
         </is>
       </c>
       <c r="B67" s="3" t="inlineStr">
         <is>
-          <t>Кронштейн</t>
+          <t>Вал ведомый</t>
         </is>
       </c>
       <c r="C67" s="3" t="inlineStr">
         <is>
-          <t>Шероховатость</t>
+          <t>Твёрдость</t>
         </is>
       </c>
       <c r="D67" s="3" t="inlineStr">
         <is>
-          <t>Ra 12,5</t>
-        </is>
-      </c>
-      <c r="E67" s="3" t="n">
-        <v>12.5</v>
-      </c>
-      <c r="F67" s="3" t="n"/>
-      <c r="G67" s="3" t="n"/>
+          <t>Твёрдость HB</t>
+        </is>
+      </c>
+      <c r="E67" s="3" t="n"/>
+      <c r="F67" s="3" t="n">
+        <v>269</v>
+      </c>
+      <c r="G67" s="3" t="n">
+        <v>302</v>
+      </c>
       <c r="H67" s="3" t="inlineStr">
         <is>
-          <t>мкм</t>
+          <t>HB</t>
         </is>
       </c>
       <c r="I67" s="3" t="inlineStr">
         <is>
-          <t>Ra</t>
+          <t>HB</t>
         </is>
       </c>
       <c r="J67" s="3" t="n"/>
@@ -6795,66 +6851,64 @@
       <c r="L67" s="3" t="inlineStr"/>
       <c r="M67" s="3" t="inlineStr">
         <is>
-          <t>Ra 12,5</t>
+          <t>269...302 HB.</t>
         </is>
       </c>
       <c r="N67" s="3" t="inlineStr">
         <is>
-          <t>Чертежи/АРМ.303412.007 Кронштейн.pdf, стр. 1</t>
+          <t>Чертежи/Вал_изм3.pdf, стр. 1</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="3" t="inlineStr">
         <is>
-          <t>АРМ.303412.007</t>
+          <t>АРМ.303411.201</t>
         </is>
       </c>
       <c r="B68" s="3" t="inlineStr">
         <is>
-          <t>Кронштейн</t>
+          <t>Вал ведомый</t>
         </is>
       </c>
       <c r="C68" s="3" t="inlineStr">
         <is>
-          <t>Шероховатость</t>
+          <t>Термообработка</t>
         </is>
       </c>
       <c r="D68" s="3" t="inlineStr">
         <is>
-          <t>Ra 25</t>
-        </is>
-      </c>
-      <c r="E68" s="3" t="n">
-        <v>25</v>
-      </c>
-      <c r="F68" s="3" t="n"/>
-      <c r="G68" s="3" t="n"/>
+          <t>Закалка ТВЧ</t>
+        </is>
+      </c>
+      <c r="E68" s="3" t="n"/>
+      <c r="F68" s="3" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="G68" s="3" t="n">
+        <v>2</v>
+      </c>
       <c r="H68" s="3" t="inlineStr">
         <is>
-          <t>мкм</t>
+          <t>мм</t>
         </is>
       </c>
       <c r="I68" s="3" t="inlineStr">
         <is>
-          <t>Ra</t>
+          <t>Закалка ТВЧ</t>
         </is>
       </c>
       <c r="J68" s="3" t="n"/>
-      <c r="K68" s="3" t="inlineStr">
-        <is>
-          <t>да</t>
-        </is>
-      </c>
+      <c r="K68" s="3" t="inlineStr"/>
       <c r="L68" s="3" t="inlineStr"/>
       <c r="M68" s="3" t="inlineStr">
         <is>
-          <t>√Ra 25 (√)</t>
+          <t>Поверхности Б закалить ТВЧ h 1,5...2,0 мм, 48...53 HRC.</t>
         </is>
       </c>
       <c r="N68" s="3" t="inlineStr">
         <is>
-          <t>Чертежи/АРМ.303412.007 Кронштейн.pdf, стр. 1</t>
+          <t>Чертежи/Вал_изм3.pdf, стр. 1</t>
         </is>
       </c>
     </row>
@@ -6876,32 +6930,36 @@
       </c>
       <c r="D69" s="3" t="inlineStr">
         <is>
-          <t>Твёрдость HB</t>
+          <t>Твёрдость HRC</t>
         </is>
       </c>
       <c r="E69" s="3" t="n"/>
       <c r="F69" s="3" t="n">
-        <v>269</v>
+        <v>48</v>
       </c>
       <c r="G69" s="3" t="n">
-        <v>302</v>
+        <v>53</v>
       </c>
       <c r="H69" s="3" t="inlineStr">
         <is>
-          <t>HB</t>
+          <t>HRC</t>
         </is>
       </c>
       <c r="I69" s="3" t="inlineStr">
         <is>
-          <t>HB</t>
+          <t>HRC</t>
         </is>
       </c>
       <c r="J69" s="3" t="n"/>
       <c r="K69" s="3" t="inlineStr"/>
-      <c r="L69" s="3" t="inlineStr"/>
+      <c r="L69" s="3" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
       <c r="M69" s="3" t="inlineStr">
         <is>
-          <t>269...302 HB.</t>
+          <t>Поверхности Б закалить ТВЧ h 1,5...2,0 мм, 48...53 HRC.</t>
         </is>
       </c>
       <c r="N69" s="3" t="inlineStr">
@@ -6923,37 +6981,35 @@
       </c>
       <c r="C70" s="3" t="inlineStr">
         <is>
-          <t>Термообработка</t>
+          <t>Общие допуски</t>
         </is>
       </c>
       <c r="D70" s="3" t="inlineStr">
         <is>
-          <t>Закалка ТВЧ</t>
+          <t>IT14</t>
         </is>
       </c>
       <c r="E70" s="3" t="n"/>
-      <c r="F70" s="3" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="G70" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="H70" s="3" t="inlineStr">
-        <is>
-          <t>мм</t>
-        </is>
-      </c>
+      <c r="F70" s="3" t="n"/>
+      <c r="G70" s="3" t="n"/>
+      <c r="H70" s="3" t="n"/>
       <c r="I70" s="3" t="inlineStr">
         <is>
-          <t>Закалка ТВЧ</t>
-        </is>
-      </c>
-      <c r="J70" s="3" t="n"/>
-      <c r="K70" s="3" t="inlineStr"/>
+          <t>H14, h14</t>
+        </is>
+      </c>
+      <c r="J70" s="3" t="n">
+        <v>14</v>
+      </c>
+      <c r="K70" s="3" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
       <c r="L70" s="3" t="inlineStr"/>
       <c r="M70" s="3" t="inlineStr">
         <is>
-          <t>Поверхности Б закалить ТВЧ h 1,5...2,0 мм, 48...53 HRC.</t>
+          <t>Неуказанные предельные отклонения размеров: H14, h14, ±IT14/2.</t>
         </is>
       </c>
       <c r="N70" s="3" t="inlineStr">
@@ -6975,32 +7031,32 @@
       </c>
       <c r="C71" s="3" t="inlineStr">
         <is>
-          <t>Твёрдость</t>
+          <t>Допуск размера</t>
         </is>
       </c>
       <c r="D71" s="3" t="inlineStr">
         <is>
-          <t>Твёрдость HRC</t>
-        </is>
-      </c>
-      <c r="E71" s="3" t="n"/>
-      <c r="F71" s="3" t="n">
-        <v>48</v>
-      </c>
-      <c r="G71" s="3" t="n">
-        <v>53</v>
-      </c>
+          <t>Ø50k6</t>
+        </is>
+      </c>
+      <c r="E71" s="3" t="n">
+        <v>50</v>
+      </c>
+      <c r="F71" s="3" t="n"/>
+      <c r="G71" s="3" t="n"/>
       <c r="H71" s="3" t="inlineStr">
         <is>
-          <t>HRC</t>
+          <t>мм</t>
         </is>
       </c>
       <c r="I71" s="3" t="inlineStr">
         <is>
-          <t>HRC</t>
-        </is>
-      </c>
-      <c r="J71" s="3" t="n"/>
+          <t>k6</t>
+        </is>
+      </c>
+      <c r="J71" s="3" t="n">
+        <v>6</v>
+      </c>
       <c r="K71" s="3" t="inlineStr"/>
       <c r="L71" s="3" t="inlineStr">
         <is>
@@ -7009,7 +7065,7 @@
       </c>
       <c r="M71" s="3" t="inlineStr">
         <is>
-          <t>Поверхности Б закалить ТВЧ h 1,5...2,0 мм, 48...53 HRC.</t>
+          <t>Ø50k6</t>
         </is>
       </c>
       <c r="N71" s="3" t="inlineStr">
@@ -7031,35 +7087,41 @@
       </c>
       <c r="C72" s="3" t="inlineStr">
         <is>
-          <t>Общие допуски</t>
+          <t>Допуск размера</t>
         </is>
       </c>
       <c r="D72" s="3" t="inlineStr">
         <is>
-          <t>IT14</t>
-        </is>
-      </c>
-      <c r="E72" s="3" t="n"/>
+          <t>Ø45h6</t>
+        </is>
+      </c>
+      <c r="E72" s="3" t="n">
+        <v>45</v>
+      </c>
       <c r="F72" s="3" t="n"/>
       <c r="G72" s="3" t="n"/>
-      <c r="H72" s="3" t="n"/>
+      <c r="H72" s="3" t="inlineStr">
+        <is>
+          <t>мм</t>
+        </is>
+      </c>
       <c r="I72" s="3" t="inlineStr">
         <is>
-          <t>H14, h14</t>
+          <t>h6</t>
         </is>
       </c>
       <c r="J72" s="3" t="n">
-        <v>14</v>
-      </c>
-      <c r="K72" s="3" t="inlineStr">
+        <v>6</v>
+      </c>
+      <c r="K72" s="3" t="inlineStr"/>
+      <c r="L72" s="3" t="inlineStr">
         <is>
           <t>да</t>
         </is>
       </c>
-      <c r="L72" s="3" t="inlineStr"/>
       <c r="M72" s="3" t="inlineStr">
         <is>
-          <t>Неуказанные предельные отклонения размеров: H14, h14, ±IT14/2.</t>
+          <t>Ø45h6</t>
         </is>
       </c>
       <c r="N72" s="3" t="inlineStr">
@@ -7086,11 +7148,11 @@
       </c>
       <c r="D73" s="3" t="inlineStr">
         <is>
-          <t>Ø50k6</t>
+          <t>16N9</t>
         </is>
       </c>
       <c r="E73" s="3" t="n">
-        <v>50</v>
+        <v>16</v>
       </c>
       <c r="F73" s="3" t="n"/>
       <c r="G73" s="3" t="n"/>
@@ -7101,21 +7163,17 @@
       </c>
       <c r="I73" s="3" t="inlineStr">
         <is>
-          <t>k6</t>
+          <t>N9</t>
         </is>
       </c>
       <c r="J73" s="3" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="K73" s="3" t="inlineStr"/>
-      <c r="L73" s="3" t="inlineStr">
-        <is>
-          <t>да</t>
-        </is>
-      </c>
+      <c r="L73" s="3" t="inlineStr"/>
       <c r="M73" s="3" t="inlineStr">
         <is>
-          <t>Ø50k6</t>
+          <t>16N9</t>
         </is>
       </c>
       <c r="N73" s="3" t="inlineStr">
@@ -7137,32 +7195,30 @@
       </c>
       <c r="C74" s="3" t="inlineStr">
         <is>
-          <t>Допуск размера</t>
+          <t>Шероховатость</t>
         </is>
       </c>
       <c r="D74" s="3" t="inlineStr">
         <is>
-          <t>Ø45h6</t>
+          <t>Ra 0,8</t>
         </is>
       </c>
       <c r="E74" s="3" t="n">
-        <v>45</v>
+        <v>0.8</v>
       </c>
       <c r="F74" s="3" t="n"/>
       <c r="G74" s="3" t="n"/>
       <c r="H74" s="3" t="inlineStr">
         <is>
-          <t>мм</t>
+          <t>мкм</t>
         </is>
       </c>
       <c r="I74" s="3" t="inlineStr">
         <is>
-          <t>h6</t>
-        </is>
-      </c>
-      <c r="J74" s="3" t="n">
-        <v>6</v>
-      </c>
+          <t>Ra</t>
+        </is>
+      </c>
+      <c r="J74" s="3" t="n"/>
       <c r="K74" s="3" t="inlineStr"/>
       <c r="L74" s="3" t="inlineStr">
         <is>
@@ -7171,7 +7227,7 @@
       </c>
       <c r="M74" s="3" t="inlineStr">
         <is>
-          <t>Ø45h6</t>
+          <t>Ra 0,8</t>
         </is>
       </c>
       <c r="N74" s="3" t="inlineStr">
@@ -7193,37 +7249,35 @@
       </c>
       <c r="C75" s="3" t="inlineStr">
         <is>
-          <t>Допуск размера</t>
+          <t>Шероховатость</t>
         </is>
       </c>
       <c r="D75" s="3" t="inlineStr">
         <is>
-          <t>16N9</t>
+          <t>Ra 1,6</t>
         </is>
       </c>
       <c r="E75" s="3" t="n">
-        <v>16</v>
+        <v>1.6</v>
       </c>
       <c r="F75" s="3" t="n"/>
       <c r="G75" s="3" t="n"/>
       <c r="H75" s="3" t="inlineStr">
         <is>
-          <t>мм</t>
+          <t>мкм</t>
         </is>
       </c>
       <c r="I75" s="3" t="inlineStr">
         <is>
-          <t>N9</t>
-        </is>
-      </c>
-      <c r="J75" s="3" t="n">
-        <v>9</v>
-      </c>
+          <t>Ra</t>
+        </is>
+      </c>
+      <c r="J75" s="3" t="n"/>
       <c r="K75" s="3" t="inlineStr"/>
       <c r="L75" s="3" t="inlineStr"/>
       <c r="M75" s="3" t="inlineStr">
         <is>
-          <t>16N9</t>
+          <t>Ra 1,6</t>
         </is>
       </c>
       <c r="N75" s="3" t="inlineStr">
@@ -7245,27 +7299,27 @@
       </c>
       <c r="C76" s="3" t="inlineStr">
         <is>
-          <t>Шероховатость</t>
+          <t>Допуск формы/расположения</t>
         </is>
       </c>
       <c r="D76" s="3" t="inlineStr">
         <is>
-          <t>Ra 0,8</t>
+          <t>↗ биения</t>
         </is>
       </c>
       <c r="E76" s="3" t="n">
-        <v>0.8</v>
+        <v>0.016</v>
       </c>
       <c r="F76" s="3" t="n"/>
       <c r="G76" s="3" t="n"/>
       <c r="H76" s="3" t="inlineStr">
         <is>
-          <t>мкм</t>
+          <t>мм</t>
         </is>
       </c>
       <c r="I76" s="3" t="inlineStr">
         <is>
-          <t>Ra</t>
+          <t>А-Б</t>
         </is>
       </c>
       <c r="J76" s="3" t="n"/>
@@ -7277,7 +7331,7 @@
       </c>
       <c r="M76" s="3" t="inlineStr">
         <is>
-          <t>Ra 0,8</t>
+          <t>↗ 0,016 А-Б</t>
         </is>
       </c>
       <c r="N76" s="3" t="inlineStr">
@@ -7304,11 +7358,11 @@
       </c>
       <c r="D77" s="3" t="inlineStr">
         <is>
-          <t>Ra 1,6</t>
+          <t>Ra 6,3</t>
         </is>
       </c>
       <c r="E77" s="3" t="n">
-        <v>1.6</v>
+        <v>6.3</v>
       </c>
       <c r="F77" s="3" t="n"/>
       <c r="G77" s="3" t="n"/>
@@ -7323,11 +7377,15 @@
         </is>
       </c>
       <c r="J77" s="3" t="n"/>
-      <c r="K77" s="3" t="inlineStr"/>
+      <c r="K77" s="3" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
       <c r="L77" s="3" t="inlineStr"/>
       <c r="M77" s="3" t="inlineStr">
         <is>
-          <t>Ra 1,6</t>
+          <t>√Ra 6,3 (√)</t>
         </is>
       </c>
       <c r="N77" s="3" t="inlineStr">
@@ -7336,116 +7394,8 @@
         </is>
       </c>
     </row>
-    <row r="78">
-      <c r="A78" s="3" t="inlineStr">
-        <is>
-          <t>АРМ.303411.201</t>
-        </is>
-      </c>
-      <c r="B78" s="3" t="inlineStr">
-        <is>
-          <t>Вал ведомый</t>
-        </is>
-      </c>
-      <c r="C78" s="3" t="inlineStr">
-        <is>
-          <t>Допуск формы/расположения</t>
-        </is>
-      </c>
-      <c r="D78" s="3" t="inlineStr">
-        <is>
-          <t>↗ биения</t>
-        </is>
-      </c>
-      <c r="E78" s="3" t="n">
-        <v>0.016</v>
-      </c>
-      <c r="F78" s="3" t="n"/>
-      <c r="G78" s="3" t="n"/>
-      <c r="H78" s="3" t="inlineStr">
-        <is>
-          <t>мм</t>
-        </is>
-      </c>
-      <c r="I78" s="3" t="inlineStr">
-        <is>
-          <t>А-Б</t>
-        </is>
-      </c>
-      <c r="J78" s="3" t="n"/>
-      <c r="K78" s="3" t="inlineStr"/>
-      <c r="L78" s="3" t="inlineStr">
-        <is>
-          <t>да</t>
-        </is>
-      </c>
-      <c r="M78" s="3" t="inlineStr">
-        <is>
-          <t>↗ 0,016 А-Б</t>
-        </is>
-      </c>
-      <c r="N78" s="3" t="inlineStr">
-        <is>
-          <t>Чертежи/Вал_изм3.pdf, стр. 1</t>
-        </is>
-      </c>
-    </row>
-    <row r="79">
-      <c r="A79" s="3" t="inlineStr">
-        <is>
-          <t>АРМ.303411.201</t>
-        </is>
-      </c>
-      <c r="B79" s="3" t="inlineStr">
-        <is>
-          <t>Вал ведомый</t>
-        </is>
-      </c>
-      <c r="C79" s="3" t="inlineStr">
-        <is>
-          <t>Шероховатость</t>
-        </is>
-      </c>
-      <c r="D79" s="3" t="inlineStr">
-        <is>
-          <t>Ra 6,3</t>
-        </is>
-      </c>
-      <c r="E79" s="3" t="n">
-        <v>6.3</v>
-      </c>
-      <c r="F79" s="3" t="n"/>
-      <c r="G79" s="3" t="n"/>
-      <c r="H79" s="3" t="inlineStr">
-        <is>
-          <t>мкм</t>
-        </is>
-      </c>
-      <c r="I79" s="3" t="inlineStr">
-        <is>
-          <t>Ra</t>
-        </is>
-      </c>
-      <c r="J79" s="3" t="n"/>
-      <c r="K79" s="3" t="inlineStr">
-        <is>
-          <t>да</t>
-        </is>
-      </c>
-      <c r="L79" s="3" t="inlineStr"/>
-      <c r="M79" s="3" t="inlineStr">
-        <is>
-          <t>√Ra 6,3 (√)</t>
-        </is>
-      </c>
-      <c r="N79" s="3" t="inlineStr">
-        <is>
-          <t>Чертежи/Вал_изм3.pdf, стр. 1</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:N79"/>
+  <autoFilter ref="A1:N77"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -7456,7 +7406,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H25"/>
+  <dimension ref="A1:H24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -8394,12 +8344,12 @@
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
         <is>
-          <t>АРМ.303411.003</t>
+          <t>АРМ.303411.005</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>Крышка торцевая</t>
+          <t>Гайка специальная</t>
         </is>
       </c>
       <c r="C24" s="3" t="inlineStr">
@@ -8409,7 +8359,7 @@
       </c>
       <c r="D24" s="3" t="inlineStr">
         <is>
-          <t>. Покрытие Хим.Окс.прм.</t>
+          <t>Покрытие Ц9.хр.</t>
         </is>
       </c>
       <c r="E24" s="3" t="inlineStr">
@@ -8419,7 +8369,7 @@
       </c>
       <c r="F24" s="3" t="inlineStr">
         <is>
-          <t>Покрытие «Хим.Окс.прм» встречается только у этой детали комплекта — отдельный передел или кооперация, проверить наличие на площадке</t>
+          <t>Покрытие «Ц9.хр» встречается только у этой детали комплекта — отдельный передел или кооперация, проверить наличие на площадке</t>
         </is>
       </c>
       <c r="G24" s="3" t="n">
@@ -8427,52 +8377,12 @@
       </c>
       <c r="H24" s="3" t="inlineStr">
         <is>
-          <t>Чертежи/АРМ.303411.003 Крышка торцевая.pdf, стр. 1</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="3" t="inlineStr">
-        <is>
-          <t>АРМ.303411.005</t>
-        </is>
-      </c>
-      <c r="B25" s="3" t="inlineStr">
-        <is>
-          <t>Гайка специальная</t>
-        </is>
-      </c>
-      <c r="C25" s="3" t="inlineStr">
-        <is>
-          <t>Покрытие</t>
-        </is>
-      </c>
-      <c r="D25" s="3" t="inlineStr">
-        <is>
-          <t>Покрытие Ц9.хр.</t>
-        </is>
-      </c>
-      <c r="E25" s="3" t="inlineStr">
-        <is>
-          <t>rare_in_kit</t>
-        </is>
-      </c>
-      <c r="F25" s="3" t="inlineStr">
-        <is>
-          <t>Покрытие «Ц9.хр» встречается только у этой детали комплекта — отдельный передел или кооперация, проверить наличие на площадке</t>
-        </is>
-      </c>
-      <c r="G25" s="3" t="n">
-        <v>0.55</v>
-      </c>
-      <c r="H25" s="3" t="inlineStr">
-        <is>
           <t>Чертежи/АРМ.303411.005 Гайка специальная.pdf, стр. 1</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H25"/>
+  <autoFilter ref="A1:H24"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -9794,7 +9704,7 @@
       </c>
       <c r="G10" s="3" t="inlineStr">
         <is>
-          <t>Крышка торцевая</t>
+          <t>Крышка торцебоя</t>
         </is>
       </c>
       <c r="H10" s="3" t="inlineStr">
@@ -10416,13 +10326,13 @@
         </is>
       </c>
       <c r="C2" s="3" t="n">
-        <v>1</v>
+        <v>0.9</v>
       </c>
       <c r="D2" s="3" t="n">
         <v>1</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>1</v>
+        <v>0.947</v>
       </c>
       <c r="F2" s="3" t="n"/>
       <c r="G2" s="3" t="n">
@@ -10491,13 +10401,13 @@
         </is>
       </c>
       <c r="C5" s="3" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="D5" s="3" t="n">
         <v>1</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>1</v>
+        <v>0.667</v>
       </c>
       <c r="F5" s="3" t="n"/>
       <c r="G5" s="3" t="n">
@@ -10636,7 +10546,7 @@
       <c r="D11" s="3" t="n"/>
       <c r="E11" s="3" t="n"/>
       <c r="F11" s="3" t="n">
-        <v>1</v>
+        <v>0.9330000000000001</v>
       </c>
       <c r="G11" s="3" t="n">
         <v>15</v>
@@ -10678,7 +10588,7 @@
       <c r="D13" s="3" t="n"/>
       <c r="E13" s="3" t="n"/>
       <c r="F13" s="3" t="n">
-        <v>1</v>
+        <v>0.9330000000000001</v>
       </c>
       <c r="G13" s="3" t="n">
         <v>15</v>
@@ -10699,7 +10609,7 @@
       <c r="D14" s="3" t="n"/>
       <c r="E14" s="3" t="n"/>
       <c r="F14" s="3" t="n">
-        <v>1</v>
+        <v>0.867</v>
       </c>
       <c r="G14" s="3" t="n">
         <v>15</v>
@@ -10825,7 +10735,7 @@
       <c r="D20" s="3" t="n"/>
       <c r="E20" s="3" t="n"/>
       <c r="F20" s="3" t="n">
-        <v>0.625</v>
+        <v>0.375</v>
       </c>
       <c r="G20" s="3" t="n">
         <v>16</v>
@@ -10846,10 +10756,10 @@
         <v>0.987</v>
       </c>
       <c r="D21" s="3" t="n">
-        <v>0.9389999999999999</v>
+        <v>0.915</v>
       </c>
       <c r="E21" s="3" t="n">
-        <v>0.963</v>
+        <v>0.949</v>
       </c>
       <c r="F21" s="3" t="n"/>
       <c r="G21" s="3" t="n">

</xml_diff>